<commit_message>
actualizacion planificacion presupuesto y riesgos
</commit_message>
<xml_diff>
--- a/docs/Planificación/01 Backlog Detallado del Producto.xlsx
+++ b/docs/Planificación/01 Backlog Detallado del Producto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Periodo Final 2026-10\Taller de Proyectos 2\semana 1\Planner\Taller_Proyectos_2\docs\Planificación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B29ECC38-E91A-4EC2-9780-542B00805C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C908C7-A43D-4782-B12D-C0E6D8F75917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog del Producto" sheetId="1" r:id="rId1"/>
@@ -1560,11 +1560,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1583,34 +1581,44 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="25">
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1622,14 +1630,6 @@
     <dxf>
       <font>
         <color rgb="FF666699"/>
-      </font>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill patternType="none"/>
@@ -2079,14 +2079,14 @@
     </row>
     <row r="2" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="45" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="43" t="s">
         <v>312</v>
       </c>
-      <c r="E2" s="46"/>
+      <c r="E2" s="44"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="7"/>
@@ -2113,14 +2113,14 @@
     </row>
     <row r="3" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="44"/>
-      <c r="D3" s="45" t="s">
+      <c r="C3" s="42"/>
+      <c r="D3" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="46"/>
+      <c r="E3" s="44"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="7"/>
@@ -2177,25 +2177,25 @@
     </row>
     <row r="5" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="49" t="s">
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="46"/>
-      <c r="H5" s="50" t="s">
+      <c r="G5" s="44"/>
+      <c r="H5" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="48"/>
-      <c r="M5" s="48"/>
-      <c r="N5" s="46"/>
+      <c r="I5" s="46"/>
+      <c r="J5" s="46"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="44"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
@@ -2265,16 +2265,16 @@
     </row>
     <row r="7" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="40" t="s">
+      <c r="C7" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="49" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="20" t="s">
@@ -2283,23 +2283,23 @@
       <c r="G7" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="40" t="s">
+      <c r="H7" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="40" t="s">
+      <c r="I7" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J7" s="40" t="s">
+      <c r="J7" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="40"/>
-      <c r="L7" s="60" t="s">
+      <c r="K7" s="49"/>
+      <c r="L7" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="M7" s="40" t="s">
+      <c r="M7" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N7" s="40" t="s">
+      <c r="N7" s="49" t="s">
         <v>34</v>
       </c>
       <c r="O7" s="1"/>
@@ -2317,23 +2317,23 @@
     </row>
     <row r="8" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
+      <c r="B8" s="50"/>
+      <c r="C8" s="50"/>
+      <c r="D8" s="50"/>
+      <c r="E8" s="50"/>
       <c r="F8" s="20" t="s">
         <v>35</v>
       </c>
       <c r="G8" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="42"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="42"/>
-      <c r="N8" s="42"/>
+      <c r="H8" s="50"/>
+      <c r="I8" s="50"/>
+      <c r="J8" s="50"/>
+      <c r="K8" s="50"/>
+      <c r="L8" s="53"/>
+      <c r="M8" s="50"/>
+      <c r="N8" s="50"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
@@ -2349,23 +2349,23 @@
     </row>
     <row r="9" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="42"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
       <c r="F9" s="20" t="s">
         <v>37</v>
       </c>
       <c r="G9" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="42"/>
-      <c r="K9" s="42"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="42"/>
-      <c r="N9" s="42"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50"/>
+      <c r="K9" s="50"/>
+      <c r="L9" s="53"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="50"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
@@ -2381,23 +2381,23 @@
     </row>
     <row r="10" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
       <c r="F10" s="20" t="s">
         <v>39</v>
       </c>
       <c r="G10" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="41"/>
-      <c r="L10" s="62"/>
-      <c r="M10" s="41"/>
-      <c r="N10" s="41"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="51"/>
+      <c r="L10" s="54"/>
+      <c r="M10" s="51"/>
+      <c r="N10" s="51"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
@@ -2413,16 +2413,16 @@
     </row>
     <row r="11" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="40" t="s">
+      <c r="C11" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D11" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="40" t="s">
+      <c r="E11" s="49" t="s">
         <v>44</v>
       </c>
       <c r="F11" s="20" t="s">
@@ -2431,25 +2431,25 @@
       <c r="G11" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="40" t="s">
+      <c r="H11" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="40" t="s">
+      <c r="I11" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J11" s="40" t="s">
+      <c r="J11" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="K11" s="40" t="s">
+      <c r="K11" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="60" t="s">
+      <c r="L11" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="M11" s="40" t="s">
+      <c r="M11" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N11" s="40" t="s">
+      <c r="N11" s="49" t="s">
         <v>50</v>
       </c>
       <c r="O11" s="1"/>
@@ -2467,23 +2467,23 @@
     </row>
     <row r="12" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="41"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
+      <c r="B12" s="51"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="51"/>
+      <c r="E12" s="51"/>
       <c r="F12" s="20" t="s">
         <v>51</v>
       </c>
       <c r="G12" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="41"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="41"/>
-      <c r="K12" s="41"/>
-      <c r="L12" s="62"/>
-      <c r="M12" s="41"/>
-      <c r="N12" s="41"/>
+      <c r="H12" s="51"/>
+      <c r="I12" s="51"/>
+      <c r="J12" s="51"/>
+      <c r="K12" s="51"/>
+      <c r="L12" s="54"/>
+      <c r="M12" s="51"/>
+      <c r="N12" s="51"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
@@ -2499,16 +2499,16 @@
     </row>
     <row r="13" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="49" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="40" t="s">
+      <c r="C13" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="49" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="40" t="s">
+      <c r="E13" s="49" t="s">
         <v>55</v>
       </c>
       <c r="F13" s="20" t="s">
@@ -2517,25 +2517,25 @@
       <c r="G13" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="H13" s="40" t="s">
+      <c r="H13" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="I13" s="40" t="s">
+      <c r="I13" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J13" s="40" t="s">
+      <c r="J13" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="K13" s="40" t="s">
+      <c r="K13" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="L13" s="60" t="s">
+      <c r="L13" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="M13" s="40" t="s">
+      <c r="M13" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N13" s="40" t="s">
+      <c r="N13" s="49" t="s">
         <v>60</v>
       </c>
       <c r="O13" s="1"/>
@@ -2553,23 +2553,23 @@
     </row>
     <row r="14" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
+      <c r="B14" s="50"/>
+      <c r="C14" s="50"/>
+      <c r="D14" s="50"/>
+      <c r="E14" s="50"/>
       <c r="F14" s="20" t="s">
         <v>61</v>
       </c>
       <c r="G14" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="61"/>
-      <c r="M14" s="42"/>
-      <c r="N14" s="42"/>
+      <c r="H14" s="50"/>
+      <c r="I14" s="50"/>
+      <c r="J14" s="50"/>
+      <c r="K14" s="50"/>
+      <c r="L14" s="53"/>
+      <c r="M14" s="50"/>
+      <c r="N14" s="50"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
@@ -2585,23 +2585,23 @@
     </row>
     <row r="15" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
       <c r="F15" s="20" t="s">
         <v>63</v>
       </c>
       <c r="G15" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="41"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="41"/>
-      <c r="K15" s="41"/>
-      <c r="L15" s="62"/>
-      <c r="M15" s="41"/>
-      <c r="N15" s="41"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="54"/>
+      <c r="M15" s="51"/>
+      <c r="N15" s="51"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
@@ -2617,16 +2617,16 @@
     </row>
     <row r="16" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="40" t="s">
+      <c r="C16" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="49" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="40" t="s">
+      <c r="E16" s="49" t="s">
         <v>68</v>
       </c>
       <c r="F16" s="20" t="s">
@@ -2635,25 +2635,25 @@
       <c r="G16" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="40" t="s">
+      <c r="H16" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="I16" s="40" t="s">
+      <c r="I16" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J16" s="40" t="s">
+      <c r="J16" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="K16" s="40" t="s">
+      <c r="K16" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="L16" s="57" t="s">
+      <c r="L16" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="M16" s="40" t="s">
+      <c r="M16" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N16" s="40"/>
+      <c r="N16" s="49"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
@@ -2669,23 +2669,23 @@
     </row>
     <row r="17" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="42"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
+      <c r="B17" s="50"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
       <c r="F17" s="20" t="s">
         <v>74</v>
       </c>
       <c r="G17" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="H17" s="42"/>
-      <c r="I17" s="42"/>
-      <c r="J17" s="42"/>
-      <c r="K17" s="42"/>
-      <c r="L17" s="58"/>
-      <c r="M17" s="42"/>
-      <c r="N17" s="42"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="50"/>
+      <c r="J17" s="50"/>
+      <c r="K17" s="50"/>
+      <c r="L17" s="56"/>
+      <c r="M17" s="50"/>
+      <c r="N17" s="50"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
@@ -2701,23 +2701,23 @@
     </row>
     <row r="18" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="42"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
+      <c r="B18" s="50"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
       <c r="F18" s="20" t="s">
         <v>76</v>
       </c>
       <c r="G18" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="42"/>
-      <c r="L18" s="58"/>
-      <c r="M18" s="42"/>
-      <c r="N18" s="42"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
+      <c r="J18" s="50"/>
+      <c r="K18" s="50"/>
+      <c r="L18" s="56"/>
+      <c r="M18" s="50"/>
+      <c r="N18" s="50"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
@@ -2733,23 +2733,23 @@
     </row>
     <row r="19" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="41"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
+      <c r="B19" s="51"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="51"/>
+      <c r="E19" s="51"/>
       <c r="F19" s="20" t="s">
         <v>78</v>
       </c>
       <c r="G19" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="H19" s="41"/>
-      <c r="I19" s="41"/>
-      <c r="J19" s="41"/>
-      <c r="K19" s="41"/>
-      <c r="L19" s="59"/>
-      <c r="M19" s="41"/>
-      <c r="N19" s="41"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
+      <c r="L19" s="57"/>
+      <c r="M19" s="51"/>
+      <c r="N19" s="51"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
@@ -2765,16 +2765,16 @@
     </row>
     <row r="20" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="40" t="s">
+      <c r="B20" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="40" t="s">
+      <c r="C20" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="40" t="s">
+      <c r="E20" s="49" t="s">
         <v>82</v>
       </c>
       <c r="F20" s="20" t="s">
@@ -2783,25 +2783,25 @@
       <c r="G20" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="H20" s="40" t="s">
+      <c r="H20" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="I20" s="40" t="s">
+      <c r="I20" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J20" s="40" t="s">
+      <c r="J20" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="K20" s="40" t="s">
+      <c r="K20" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="L20" s="57" t="s">
+      <c r="L20" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="M20" s="40" t="s">
+      <c r="M20" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N20" s="40" t="s">
+      <c r="N20" s="49" t="s">
         <v>87</v>
       </c>
       <c r="O20" s="1"/>
@@ -2819,23 +2819,23 @@
     </row>
     <row r="21" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="42"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="42"/>
+      <c r="B21" s="50"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
       <c r="F21" s="20" t="s">
         <v>88</v>
       </c>
       <c r="G21" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="42"/>
-      <c r="I21" s="42"/>
-      <c r="J21" s="42"/>
-      <c r="K21" s="42"/>
-      <c r="L21" s="58"/>
-      <c r="M21" s="42"/>
-      <c r="N21" s="42"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="50"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="56"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="50"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
@@ -2851,23 +2851,23 @@
     </row>
     <row r="22" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="42"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
+      <c r="B22" s="50"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
       <c r="F22" s="20" t="s">
         <v>90</v>
       </c>
       <c r="G22" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42"/>
-      <c r="J22" s="42"/>
-      <c r="K22" s="42"/>
-      <c r="L22" s="58"/>
-      <c r="M22" s="42"/>
-      <c r="N22" s="42"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="50"/>
+      <c r="J22" s="50"/>
+      <c r="K22" s="50"/>
+      <c r="L22" s="56"/>
+      <c r="M22" s="50"/>
+      <c r="N22" s="50"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
@@ -2883,23 +2883,23 @@
     </row>
     <row r="23" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
+      <c r="B23" s="51"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="51"/>
       <c r="F23" s="20" t="s">
         <v>92</v>
       </c>
       <c r="G23" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="H23" s="41"/>
-      <c r="I23" s="41"/>
-      <c r="J23" s="41"/>
-      <c r="K23" s="41"/>
-      <c r="L23" s="59"/>
-      <c r="M23" s="41"/>
-      <c r="N23" s="41"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="51"/>
+      <c r="K23" s="51"/>
+      <c r="L23" s="57"/>
+      <c r="M23" s="51"/>
+      <c r="N23" s="51"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
@@ -2915,16 +2915,16 @@
     </row>
     <row r="24" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="49" t="s">
         <v>94</v>
       </c>
-      <c r="C24" s="40" t="s">
+      <c r="C24" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="D24" s="40" t="s">
+      <c r="D24" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="E24" s="40" t="s">
+      <c r="E24" s="49" t="s">
         <v>96</v>
       </c>
       <c r="F24" s="20" t="s">
@@ -2933,25 +2933,25 @@
       <c r="G24" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="H24" s="40" t="s">
+      <c r="H24" s="49" t="s">
         <v>99</v>
       </c>
-      <c r="I24" s="40" t="s">
+      <c r="I24" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J24" s="40" t="s">
+      <c r="J24" s="49" t="s">
         <v>100</v>
       </c>
-      <c r="K24" s="40" t="s">
+      <c r="K24" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="L24" s="57" t="s">
+      <c r="L24" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="M24" s="40" t="s">
+      <c r="M24" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N24" s="40" t="s">
+      <c r="N24" s="49" t="s">
         <v>101</v>
       </c>
       <c r="O24" s="1"/>
@@ -2969,23 +2969,23 @@
     </row>
     <row r="25" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="50"/>
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
       <c r="F25" s="20" t="s">
         <v>102</v>
       </c>
       <c r="G25" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="42"/>
-      <c r="I25" s="42"/>
-      <c r="J25" s="42"/>
-      <c r="K25" s="42"/>
-      <c r="L25" s="58"/>
-      <c r="M25" s="42"/>
-      <c r="N25" s="42"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="56"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="50"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
@@ -3001,23 +3001,23 @@
     </row>
     <row r="26" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
-      <c r="B26" s="42"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
+      <c r="B26" s="50"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="50"/>
+      <c r="E26" s="50"/>
       <c r="F26" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G26" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="H26" s="42"/>
-      <c r="I26" s="42"/>
-      <c r="J26" s="42"/>
-      <c r="K26" s="42"/>
-      <c r="L26" s="58"/>
-      <c r="M26" s="42"/>
-      <c r="N26" s="42"/>
+      <c r="H26" s="50"/>
+      <c r="I26" s="50"/>
+      <c r="J26" s="50"/>
+      <c r="K26" s="50"/>
+      <c r="L26" s="56"/>
+      <c r="M26" s="50"/>
+      <c r="N26" s="50"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
@@ -3033,23 +3033,23 @@
     </row>
     <row r="27" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
-      <c r="B27" s="41"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
       <c r="F27" s="20" t="s">
         <v>106</v>
       </c>
       <c r="G27" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="H27" s="41"/>
-      <c r="I27" s="41"/>
-      <c r="J27" s="41"/>
-      <c r="K27" s="41"/>
-      <c r="L27" s="59"/>
-      <c r="M27" s="41"/>
-      <c r="N27" s="41"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="51"/>
+      <c r="L27" s="57"/>
+      <c r="M27" s="51"/>
+      <c r="N27" s="51"/>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
@@ -3065,16 +3065,16 @@
     </row>
     <row r="28" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
-      <c r="B28" s="40" t="s">
+      <c r="B28" s="49" t="s">
         <v>108</v>
       </c>
-      <c r="C28" s="40" t="s">
+      <c r="C28" s="49" t="s">
         <v>66</v>
       </c>
-      <c r="D28" s="40" t="s">
+      <c r="D28" s="49" t="s">
         <v>109</v>
       </c>
-      <c r="E28" s="40" t="s">
+      <c r="E28" s="49" t="s">
         <v>110</v>
       </c>
       <c r="F28" s="20" t="s">
@@ -3083,25 +3083,25 @@
       <c r="G28" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="H28" s="40" t="s">
+      <c r="H28" s="49" t="s">
         <v>113</v>
       </c>
-      <c r="I28" s="40" t="s">
+      <c r="I28" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J28" s="40" t="s">
+      <c r="J28" s="49" t="s">
         <v>114</v>
       </c>
-      <c r="K28" s="40" t="s">
+      <c r="K28" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="L28" s="57" t="s">
+      <c r="L28" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="M28" s="40" t="s">
+      <c r="M28" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N28" s="40" t="s">
+      <c r="N28" s="49" t="s">
         <v>115</v>
       </c>
       <c r="O28" s="1"/>
@@ -3119,23 +3119,23 @@
     </row>
     <row r="29" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
-      <c r="B29" s="42"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="42"/>
+      <c r="B29" s="50"/>
+      <c r="C29" s="50"/>
+      <c r="D29" s="50"/>
+      <c r="E29" s="50"/>
       <c r="F29" s="20" t="s">
         <v>116</v>
       </c>
       <c r="G29" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="H29" s="42"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="42"/>
-      <c r="K29" s="42"/>
-      <c r="L29" s="58"/>
-      <c r="M29" s="42"/>
-      <c r="N29" s="42"/>
+      <c r="H29" s="50"/>
+      <c r="I29" s="50"/>
+      <c r="J29" s="50"/>
+      <c r="K29" s="50"/>
+      <c r="L29" s="56"/>
+      <c r="M29" s="50"/>
+      <c r="N29" s="50"/>
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
@@ -3151,23 +3151,23 @@
     </row>
     <row r="30" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
-      <c r="B30" s="41"/>
-      <c r="C30" s="41"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
+      <c r="B30" s="51"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
       <c r="F30" s="20" t="s">
         <v>118</v>
       </c>
       <c r="G30" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="H30" s="41"/>
-      <c r="I30" s="41"/>
-      <c r="J30" s="41"/>
-      <c r="K30" s="41"/>
-      <c r="L30" s="59"/>
-      <c r="M30" s="41"/>
-      <c r="N30" s="41"/>
+      <c r="H30" s="51"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="51"/>
+      <c r="K30" s="51"/>
+      <c r="L30" s="57"/>
+      <c r="M30" s="51"/>
+      <c r="N30" s="51"/>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
@@ -3183,16 +3183,16 @@
     </row>
     <row r="31" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
-      <c r="B31" s="40" t="s">
+      <c r="B31" s="49" t="s">
         <v>120</v>
       </c>
-      <c r="C31" s="40" t="s">
+      <c r="C31" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D31" s="40" t="s">
+      <c r="D31" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="E31" s="40" t="s">
+      <c r="E31" s="49" t="s">
         <v>122</v>
       </c>
       <c r="F31" s="20" t="s">
@@ -3201,25 +3201,25 @@
       <c r="G31" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="H31" s="40" t="s">
+      <c r="H31" s="49" t="s">
         <v>125</v>
       </c>
-      <c r="I31" s="40" t="s">
+      <c r="I31" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J31" s="40" t="s">
+      <c r="J31" s="49" t="s">
         <v>126</v>
       </c>
-      <c r="K31" s="40" t="s">
+      <c r="K31" s="49" t="s">
         <v>127</v>
       </c>
-      <c r="L31" s="54" t="s">
+      <c r="L31" s="58" t="s">
         <v>183</v>
       </c>
-      <c r="M31" s="40" t="s">
+      <c r="M31" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N31" s="40" t="s">
+      <c r="N31" s="49" t="s">
         <v>128</v>
       </c>
       <c r="O31" s="1"/>
@@ -3237,23 +3237,23 @@
     </row>
     <row r="32" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
-      <c r="B32" s="42"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="42"/>
-      <c r="E32" s="42"/>
+      <c r="B32" s="50"/>
+      <c r="C32" s="50"/>
+      <c r="D32" s="50"/>
+      <c r="E32" s="50"/>
       <c r="F32" s="20" t="s">
         <v>129</v>
       </c>
       <c r="G32" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="H32" s="42"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="42"/>
-      <c r="K32" s="42"/>
-      <c r="L32" s="55"/>
-      <c r="M32" s="42"/>
-      <c r="N32" s="42"/>
+      <c r="H32" s="50"/>
+      <c r="I32" s="50"/>
+      <c r="J32" s="50"/>
+      <c r="K32" s="50"/>
+      <c r="L32" s="59"/>
+      <c r="M32" s="50"/>
+      <c r="N32" s="50"/>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
@@ -3269,23 +3269,23 @@
     </row>
     <row r="33" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
+      <c r="B33" s="51"/>
+      <c r="C33" s="51"/>
+      <c r="D33" s="51"/>
+      <c r="E33" s="51"/>
       <c r="F33" s="20" t="s">
         <v>131</v>
       </c>
       <c r="G33" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-      <c r="J33" s="41"/>
-      <c r="K33" s="41"/>
-      <c r="L33" s="56"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
+      <c r="H33" s="51"/>
+      <c r="I33" s="51"/>
+      <c r="J33" s="51"/>
+      <c r="K33" s="51"/>
+      <c r="L33" s="60"/>
+      <c r="M33" s="51"/>
+      <c r="N33" s="51"/>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
@@ -3301,16 +3301,16 @@
     </row>
     <row r="34" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
-      <c r="B34" s="40" t="s">
+      <c r="B34" s="49" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="40" t="s">
+      <c r="C34" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D34" s="40" t="s">
+      <c r="D34" s="49" t="s">
         <v>134</v>
       </c>
-      <c r="E34" s="40" t="s">
+      <c r="E34" s="49" t="s">
         <v>135</v>
       </c>
       <c r="F34" s="20" t="s">
@@ -3319,25 +3319,25 @@
       <c r="G34" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="H34" s="40" t="s">
+      <c r="H34" s="49" t="s">
         <v>138</v>
       </c>
-      <c r="I34" s="40" t="s">
+      <c r="I34" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="40" t="s">
+      <c r="J34" s="49" t="s">
         <v>139</v>
       </c>
-      <c r="K34" s="40" t="s">
+      <c r="K34" s="49" t="s">
         <v>140</v>
       </c>
-      <c r="L34" s="54" t="s">
+      <c r="L34" s="58" t="s">
         <v>183</v>
       </c>
-      <c r="M34" s="40" t="s">
+      <c r="M34" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N34" s="40" t="s">
+      <c r="N34" s="49" t="s">
         <v>141</v>
       </c>
       <c r="O34" s="1"/>
@@ -3355,23 +3355,23 @@
     </row>
     <row r="35" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
-      <c r="B35" s="42"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="42"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="50"/>
       <c r="F35" s="20" t="s">
         <v>142</v>
       </c>
       <c r="G35" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="H35" s="42"/>
-      <c r="I35" s="42"/>
-      <c r="J35" s="42"/>
-      <c r="K35" s="42"/>
-      <c r="L35" s="55"/>
-      <c r="M35" s="42"/>
-      <c r="N35" s="42"/>
+      <c r="H35" s="50"/>
+      <c r="I35" s="50"/>
+      <c r="J35" s="50"/>
+      <c r="K35" s="50"/>
+      <c r="L35" s="59"/>
+      <c r="M35" s="50"/>
+      <c r="N35" s="50"/>
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
@@ -3387,23 +3387,23 @@
     </row>
     <row r="36" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
-      <c r="B36" s="42"/>
-      <c r="C36" s="42"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="42"/>
+      <c r="B36" s="50"/>
+      <c r="C36" s="50"/>
+      <c r="D36" s="50"/>
+      <c r="E36" s="50"/>
       <c r="F36" s="20" t="s">
         <v>144</v>
       </c>
       <c r="G36" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="55"/>
-      <c r="M36" s="42"/>
-      <c r="N36" s="42"/>
+      <c r="H36" s="50"/>
+      <c r="I36" s="50"/>
+      <c r="J36" s="50"/>
+      <c r="K36" s="50"/>
+      <c r="L36" s="59"/>
+      <c r="M36" s="50"/>
+      <c r="N36" s="50"/>
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
@@ -3419,23 +3419,23 @@
     </row>
     <row r="37" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
-      <c r="B37" s="41"/>
-      <c r="C37" s="41"/>
-      <c r="D37" s="41"/>
-      <c r="E37" s="41"/>
+      <c r="B37" s="51"/>
+      <c r="C37" s="51"/>
+      <c r="D37" s="51"/>
+      <c r="E37" s="51"/>
       <c r="F37" s="20" t="s">
         <v>146</v>
       </c>
       <c r="G37" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="H37" s="41"/>
-      <c r="I37" s="41"/>
-      <c r="J37" s="41"/>
-      <c r="K37" s="41"/>
-      <c r="L37" s="56"/>
-      <c r="M37" s="41"/>
-      <c r="N37" s="41"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="51"/>
+      <c r="J37" s="51"/>
+      <c r="K37" s="51"/>
+      <c r="L37" s="60"/>
+      <c r="M37" s="51"/>
+      <c r="N37" s="51"/>
       <c r="O37" s="1"/>
       <c r="P37" s="1"/>
       <c r="Q37" s="1"/>
@@ -3451,16 +3451,16 @@
     </row>
     <row r="38" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
-      <c r="B38" s="40" t="s">
+      <c r="B38" s="49" t="s">
         <v>148</v>
       </c>
-      <c r="C38" s="40" t="s">
+      <c r="C38" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D38" s="40" t="s">
+      <c r="D38" s="49" t="s">
         <v>149</v>
       </c>
-      <c r="E38" s="40" t="s">
+      <c r="E38" s="49" t="s">
         <v>150</v>
       </c>
       <c r="F38" s="20" t="s">
@@ -3469,25 +3469,25 @@
       <c r="G38" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="H38" s="40" t="s">
+      <c r="H38" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="I38" s="40" t="s">
+      <c r="I38" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J38" s="40" t="s">
+      <c r="J38" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="K38" s="40" t="s">
+      <c r="K38" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="L38" s="54" t="s">
+      <c r="L38" s="58" t="s">
         <v>183</v>
       </c>
-      <c r="M38" s="40" t="s">
+      <c r="M38" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N38" s="40" t="s">
+      <c r="N38" s="49" t="s">
         <v>155</v>
       </c>
       <c r="O38" s="1"/>
@@ -3505,23 +3505,23 @@
     </row>
     <row r="39" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
-      <c r="B39" s="42"/>
-      <c r="C39" s="42"/>
-      <c r="D39" s="42"/>
-      <c r="E39" s="42"/>
+      <c r="B39" s="50"/>
+      <c r="C39" s="50"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="50"/>
       <c r="F39" s="20" t="s">
         <v>156</v>
       </c>
       <c r="G39" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="H39" s="42"/>
-      <c r="I39" s="42"/>
-      <c r="J39" s="42"/>
-      <c r="K39" s="42"/>
-      <c r="L39" s="55"/>
-      <c r="M39" s="42"/>
-      <c r="N39" s="42"/>
+      <c r="H39" s="50"/>
+      <c r="I39" s="50"/>
+      <c r="J39" s="50"/>
+      <c r="K39" s="50"/>
+      <c r="L39" s="59"/>
+      <c r="M39" s="50"/>
+      <c r="N39" s="50"/>
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
@@ -3537,23 +3537,23 @@
     </row>
     <row r="40" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
-      <c r="B40" s="41"/>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
+      <c r="B40" s="51"/>
+      <c r="C40" s="51"/>
+      <c r="D40" s="51"/>
+      <c r="E40" s="51"/>
       <c r="F40" s="20" t="s">
         <v>158</v>
       </c>
       <c r="G40" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="H40" s="41"/>
-      <c r="I40" s="41"/>
-      <c r="J40" s="41"/>
-      <c r="K40" s="41"/>
-      <c r="L40" s="56"/>
-      <c r="M40" s="41"/>
-      <c r="N40" s="41"/>
+      <c r="H40" s="51"/>
+      <c r="I40" s="51"/>
+      <c r="J40" s="51"/>
+      <c r="K40" s="51"/>
+      <c r="L40" s="60"/>
+      <c r="M40" s="51"/>
+      <c r="N40" s="51"/>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
@@ -3569,16 +3569,16 @@
     </row>
     <row r="41" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1"/>
-      <c r="B41" s="40" t="s">
+      <c r="B41" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="C41" s="40" t="s">
+      <c r="C41" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="D41" s="40" t="s">
+      <c r="D41" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="E41" s="40" t="s">
+      <c r="E41" s="49" t="s">
         <v>163</v>
       </c>
       <c r="F41" s="20" t="s">
@@ -3587,25 +3587,25 @@
       <c r="G41" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="H41" s="40" t="s">
+      <c r="H41" s="49" t="s">
         <v>166</v>
       </c>
-      <c r="I41" s="40" t="s">
+      <c r="I41" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J41" s="40" t="s">
+      <c r="J41" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="K41" s="40" t="s">
+      <c r="K41" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="L41" s="54" t="s">
+      <c r="L41" s="58" t="s">
         <v>183</v>
       </c>
-      <c r="M41" s="40" t="s">
+      <c r="M41" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N41" s="40" t="s">
+      <c r="N41" s="49" t="s">
         <v>169</v>
       </c>
       <c r="O41" s="1"/>
@@ -3623,23 +3623,23 @@
     </row>
     <row r="42" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1"/>
-      <c r="B42" s="42"/>
-      <c r="C42" s="42"/>
-      <c r="D42" s="42"/>
-      <c r="E42" s="42"/>
+      <c r="B42" s="50"/>
+      <c r="C42" s="50"/>
+      <c r="D42" s="50"/>
+      <c r="E42" s="50"/>
       <c r="F42" s="20" t="s">
         <v>170</v>
       </c>
       <c r="G42" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
-      <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="55"/>
-      <c r="M42" s="42"/>
-      <c r="N42" s="42"/>
+      <c r="H42" s="50"/>
+      <c r="I42" s="50"/>
+      <c r="J42" s="50"/>
+      <c r="K42" s="50"/>
+      <c r="L42" s="59"/>
+      <c r="M42" s="50"/>
+      <c r="N42" s="50"/>
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
@@ -3655,23 +3655,23 @@
     </row>
     <row r="43" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1"/>
-      <c r="B43" s="41"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="41"/>
-      <c r="E43" s="41"/>
+      <c r="B43" s="51"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="51"/>
+      <c r="E43" s="51"/>
       <c r="F43" s="20" t="s">
         <v>172</v>
       </c>
       <c r="G43" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="H43" s="41"/>
-      <c r="I43" s="41"/>
-      <c r="J43" s="41"/>
-      <c r="K43" s="41"/>
-      <c r="L43" s="56"/>
-      <c r="M43" s="41"/>
-      <c r="N43" s="41"/>
+      <c r="H43" s="51"/>
+      <c r="I43" s="51"/>
+      <c r="J43" s="51"/>
+      <c r="K43" s="51"/>
+      <c r="L43" s="60"/>
+      <c r="M43" s="51"/>
+      <c r="N43" s="51"/>
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
@@ -3687,16 +3687,16 @@
     </row>
     <row r="44" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1"/>
-      <c r="B44" s="40" t="s">
+      <c r="B44" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="C44" s="40" t="s">
+      <c r="C44" s="49" t="s">
         <v>175</v>
       </c>
-      <c r="D44" s="40" t="s">
+      <c r="D44" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="E44" s="40" t="s">
+      <c r="E44" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F44" s="20" t="s">
@@ -3705,25 +3705,25 @@
       <c r="G44" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="H44" s="40" t="s">
+      <c r="H44" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="I44" s="40" t="s">
+      <c r="I44" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J44" s="40" t="s">
+      <c r="J44" s="49" t="s">
         <v>181</v>
       </c>
-      <c r="K44" s="40" t="s">
+      <c r="K44" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="L44" s="51" t="s">
+      <c r="L44" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M44" s="40" t="s">
+      <c r="M44" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N44" s="40" t="s">
+      <c r="N44" s="49" t="s">
         <v>184</v>
       </c>
       <c r="O44" s="1"/>
@@ -3741,23 +3741,23 @@
     </row>
     <row r="45" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1"/>
-      <c r="B45" s="42"/>
-      <c r="C45" s="42"/>
-      <c r="D45" s="42"/>
-      <c r="E45" s="42"/>
+      <c r="B45" s="50"/>
+      <c r="C45" s="50"/>
+      <c r="D45" s="50"/>
+      <c r="E45" s="50"/>
       <c r="F45" s="20" t="s">
         <v>185</v>
       </c>
       <c r="G45" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="H45" s="42"/>
-      <c r="I45" s="42"/>
-      <c r="J45" s="42"/>
-      <c r="K45" s="42"/>
-      <c r="L45" s="52"/>
-      <c r="M45" s="42"/>
-      <c r="N45" s="42"/>
+      <c r="H45" s="50"/>
+      <c r="I45" s="50"/>
+      <c r="J45" s="50"/>
+      <c r="K45" s="50"/>
+      <c r="L45" s="62"/>
+      <c r="M45" s="50"/>
+      <c r="N45" s="50"/>
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
@@ -3773,23 +3773,23 @@
     </row>
     <row r="46" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1"/>
-      <c r="B46" s="41"/>
-      <c r="C46" s="41"/>
-      <c r="D46" s="41"/>
-      <c r="E46" s="41"/>
+      <c r="B46" s="51"/>
+      <c r="C46" s="51"/>
+      <c r="D46" s="51"/>
+      <c r="E46" s="51"/>
       <c r="F46" s="20" t="s">
         <v>187</v>
       </c>
       <c r="G46" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="H46" s="41"/>
-      <c r="I46" s="41"/>
-      <c r="J46" s="41"/>
-      <c r="K46" s="41"/>
-      <c r="L46" s="53"/>
-      <c r="M46" s="41"/>
-      <c r="N46" s="41"/>
+      <c r="H46" s="51"/>
+      <c r="I46" s="51"/>
+      <c r="J46" s="51"/>
+      <c r="K46" s="51"/>
+      <c r="L46" s="63"/>
+      <c r="M46" s="51"/>
+      <c r="N46" s="51"/>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
@@ -3805,16 +3805,16 @@
     </row>
     <row r="47" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1"/>
-      <c r="B47" s="40" t="s">
+      <c r="B47" s="49" t="s">
         <v>189</v>
       </c>
-      <c r="C47" s="40" t="s">
+      <c r="C47" s="49" t="s">
         <v>175</v>
       </c>
-      <c r="D47" s="40" t="s">
+      <c r="D47" s="49" t="s">
         <v>190</v>
       </c>
-      <c r="E47" s="40" t="s">
+      <c r="E47" s="49" t="s">
         <v>191</v>
       </c>
       <c r="F47" s="20" t="s">
@@ -3823,25 +3823,25 @@
       <c r="G47" s="20" t="s">
         <v>193</v>
       </c>
-      <c r="H47" s="40" t="s">
+      <c r="H47" s="49" t="s">
         <v>194</v>
       </c>
-      <c r="I47" s="40" t="s">
+      <c r="I47" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J47" s="40" t="s">
+      <c r="J47" s="49" t="s">
         <v>195</v>
       </c>
-      <c r="K47" s="40" t="s">
+      <c r="K47" s="49" t="s">
         <v>196</v>
       </c>
-      <c r="L47" s="51" t="s">
+      <c r="L47" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M47" s="40" t="s">
+      <c r="M47" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N47" s="40" t="s">
+      <c r="N47" s="49" t="s">
         <v>197</v>
       </c>
       <c r="O47" s="1"/>
@@ -3859,23 +3859,23 @@
     </row>
     <row r="48" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1"/>
-      <c r="B48" s="42"/>
-      <c r="C48" s="42"/>
-      <c r="D48" s="42"/>
-      <c r="E48" s="42"/>
+      <c r="B48" s="50"/>
+      <c r="C48" s="50"/>
+      <c r="D48" s="50"/>
+      <c r="E48" s="50"/>
       <c r="F48" s="20" t="s">
         <v>198</v>
       </c>
       <c r="G48" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="H48" s="42"/>
-      <c r="I48" s="42"/>
-      <c r="J48" s="42"/>
-      <c r="K48" s="42"/>
-      <c r="L48" s="52"/>
-      <c r="M48" s="42"/>
-      <c r="N48" s="42"/>
+      <c r="H48" s="50"/>
+      <c r="I48" s="50"/>
+      <c r="J48" s="50"/>
+      <c r="K48" s="50"/>
+      <c r="L48" s="62"/>
+      <c r="M48" s="50"/>
+      <c r="N48" s="50"/>
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
@@ -3891,23 +3891,23 @@
     </row>
     <row r="49" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1"/>
-      <c r="B49" s="41"/>
-      <c r="C49" s="41"/>
-      <c r="D49" s="41"/>
-      <c r="E49" s="41"/>
+      <c r="B49" s="51"/>
+      <c r="C49" s="51"/>
+      <c r="D49" s="51"/>
+      <c r="E49" s="51"/>
       <c r="F49" s="20" t="s">
         <v>200</v>
       </c>
       <c r="G49" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="H49" s="41"/>
-      <c r="I49" s="41"/>
-      <c r="J49" s="41"/>
-      <c r="K49" s="41"/>
-      <c r="L49" s="53"/>
-      <c r="M49" s="41"/>
-      <c r="N49" s="41"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="51"/>
+      <c r="K49" s="51"/>
+      <c r="L49" s="63"/>
+      <c r="M49" s="51"/>
+      <c r="N49" s="51"/>
       <c r="O49" s="1"/>
       <c r="P49" s="1"/>
       <c r="Q49" s="1"/>
@@ -3923,16 +3923,16 @@
     </row>
     <row r="50" spans="1:26" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1"/>
-      <c r="B50" s="40" t="s">
+      <c r="B50" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="C50" s="40" t="s">
+      <c r="C50" s="49" t="s">
         <v>203</v>
       </c>
-      <c r="D50" s="40" t="s">
+      <c r="D50" s="49" t="s">
         <v>204</v>
       </c>
-      <c r="E50" s="40" t="s">
+      <c r="E50" s="49" t="s">
         <v>205</v>
       </c>
       <c r="F50" s="20" t="s">
@@ -3941,25 +3941,25 @@
       <c r="G50" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="H50" s="40" t="s">
+      <c r="H50" s="49" t="s">
         <v>208</v>
       </c>
-      <c r="I50" s="40" t="s">
+      <c r="I50" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J50" s="40" t="s">
+      <c r="J50" s="49" t="s">
         <v>209</v>
       </c>
-      <c r="K50" s="40" t="s">
+      <c r="K50" s="49" t="s">
         <v>210</v>
       </c>
-      <c r="L50" s="51" t="s">
+      <c r="L50" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M50" s="40" t="s">
+      <c r="M50" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N50" s="40" t="s">
+      <c r="N50" s="49" t="s">
         <v>211</v>
       </c>
       <c r="O50" s="1"/>
@@ -3977,23 +3977,23 @@
     </row>
     <row r="51" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1"/>
-      <c r="B51" s="41"/>
-      <c r="C51" s="41"/>
-      <c r="D51" s="41"/>
-      <c r="E51" s="41"/>
+      <c r="B51" s="51"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="51"/>
+      <c r="E51" s="51"/>
       <c r="F51" s="20" t="s">
         <v>212</v>
       </c>
       <c r="G51" s="20" t="s">
         <v>213</v>
       </c>
-      <c r="H51" s="41"/>
-      <c r="I51" s="41"/>
-      <c r="J51" s="41"/>
-      <c r="K51" s="41"/>
-      <c r="L51" s="53"/>
-      <c r="M51" s="41"/>
-      <c r="N51" s="41"/>
+      <c r="H51" s="51"/>
+      <c r="I51" s="51"/>
+      <c r="J51" s="51"/>
+      <c r="K51" s="51"/>
+      <c r="L51" s="63"/>
+      <c r="M51" s="51"/>
+      <c r="N51" s="51"/>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
@@ -4009,16 +4009,16 @@
     </row>
     <row r="52" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1"/>
-      <c r="B52" s="40" t="s">
+      <c r="B52" s="49" t="s">
         <v>214</v>
       </c>
-      <c r="C52" s="40" t="s">
+      <c r="C52" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="D52" s="40" t="s">
+      <c r="D52" s="49" t="s">
         <v>216</v>
       </c>
-      <c r="E52" s="40" t="s">
+      <c r="E52" s="49" t="s">
         <v>217</v>
       </c>
       <c r="F52" s="20" t="s">
@@ -4027,25 +4027,25 @@
       <c r="G52" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="H52" s="40" t="s">
+      <c r="H52" s="49" t="s">
         <v>220</v>
       </c>
-      <c r="I52" s="40" t="s">
+      <c r="I52" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J52" s="40" t="s">
+      <c r="J52" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="K52" s="40" t="s">
+      <c r="K52" s="49" t="s">
         <v>222</v>
       </c>
-      <c r="L52" s="51" t="s">
+      <c r="L52" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M52" s="40" t="s">
+      <c r="M52" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N52" s="40" t="s">
+      <c r="N52" s="49" t="s">
         <v>223</v>
       </c>
       <c r="O52" s="1"/>
@@ -4063,23 +4063,23 @@
     </row>
     <row r="53" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1"/>
-      <c r="B53" s="42"/>
-      <c r="C53" s="42"/>
-      <c r="D53" s="42"/>
-      <c r="E53" s="42"/>
+      <c r="B53" s="50"/>
+      <c r="C53" s="50"/>
+      <c r="D53" s="50"/>
+      <c r="E53" s="50"/>
       <c r="F53" s="20" t="s">
         <v>224</v>
       </c>
       <c r="G53" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="H53" s="42"/>
-      <c r="I53" s="42"/>
-      <c r="J53" s="42"/>
-      <c r="K53" s="42"/>
-      <c r="L53" s="52"/>
-      <c r="M53" s="42"/>
-      <c r="N53" s="42"/>
+      <c r="H53" s="50"/>
+      <c r="I53" s="50"/>
+      <c r="J53" s="50"/>
+      <c r="K53" s="50"/>
+      <c r="L53" s="62"/>
+      <c r="M53" s="50"/>
+      <c r="N53" s="50"/>
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
@@ -4095,23 +4095,23 @@
     </row>
     <row r="54" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1"/>
-      <c r="B54" s="41"/>
-      <c r="C54" s="41"/>
-      <c r="D54" s="41"/>
-      <c r="E54" s="41"/>
+      <c r="B54" s="51"/>
+      <c r="C54" s="51"/>
+      <c r="D54" s="51"/>
+      <c r="E54" s="51"/>
       <c r="F54" s="20" t="s">
         <v>226</v>
       </c>
       <c r="G54" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="H54" s="41"/>
-      <c r="I54" s="41"/>
-      <c r="J54" s="41"/>
-      <c r="K54" s="41"/>
-      <c r="L54" s="53"/>
-      <c r="M54" s="41"/>
-      <c r="N54" s="41"/>
+      <c r="H54" s="51"/>
+      <c r="I54" s="51"/>
+      <c r="J54" s="51"/>
+      <c r="K54" s="51"/>
+      <c r="L54" s="63"/>
+      <c r="M54" s="51"/>
+      <c r="N54" s="51"/>
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
@@ -4127,16 +4127,16 @@
     </row>
     <row r="55" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1"/>
-      <c r="B55" s="40" t="s">
+      <c r="B55" s="49" t="s">
         <v>228</v>
       </c>
-      <c r="C55" s="40" t="s">
+      <c r="C55" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="D55" s="40" t="s">
+      <c r="D55" s="49" t="s">
         <v>229</v>
       </c>
-      <c r="E55" s="40" t="s">
+      <c r="E55" s="49" t="s">
         <v>230</v>
       </c>
       <c r="F55" s="20" t="s">
@@ -4145,25 +4145,25 @@
       <c r="G55" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="H55" s="40" t="s">
+      <c r="H55" s="49" t="s">
         <v>233</v>
       </c>
-      <c r="I55" s="40" t="s">
+      <c r="I55" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J55" s="40" t="s">
+      <c r="J55" s="49" t="s">
         <v>234</v>
       </c>
-      <c r="K55" s="40" t="s">
+      <c r="K55" s="49" t="s">
         <v>235</v>
       </c>
-      <c r="L55" s="51" t="s">
+      <c r="L55" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M55" s="40" t="s">
+      <c r="M55" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N55" s="40" t="s">
+      <c r="N55" s="49" t="s">
         <v>236</v>
       </c>
       <c r="O55" s="1"/>
@@ -4181,23 +4181,23 @@
     </row>
     <row r="56" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1"/>
-      <c r="B56" s="41"/>
-      <c r="C56" s="41"/>
-      <c r="D56" s="41"/>
-      <c r="E56" s="41"/>
+      <c r="B56" s="51"/>
+      <c r="C56" s="51"/>
+      <c r="D56" s="51"/>
+      <c r="E56" s="51"/>
       <c r="F56" s="20" t="s">
         <v>237</v>
       </c>
       <c r="G56" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H56" s="41"/>
-      <c r="I56" s="41"/>
-      <c r="J56" s="41"/>
-      <c r="K56" s="41"/>
-      <c r="L56" s="53"/>
-      <c r="M56" s="41"/>
-      <c r="N56" s="41"/>
+      <c r="H56" s="51"/>
+      <c r="I56" s="51"/>
+      <c r="J56" s="51"/>
+      <c r="K56" s="51"/>
+      <c r="L56" s="63"/>
+      <c r="M56" s="51"/>
+      <c r="N56" s="51"/>
       <c r="O56" s="1"/>
       <c r="P56" s="1"/>
       <c r="Q56" s="1"/>
@@ -4213,16 +4213,16 @@
     </row>
     <row r="57" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1"/>
-      <c r="B57" s="40" t="s">
+      <c r="B57" s="49" t="s">
         <v>239</v>
       </c>
-      <c r="C57" s="40" t="s">
+      <c r="C57" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="D57" s="40" t="s">
+      <c r="D57" s="49" t="s">
         <v>240</v>
       </c>
-      <c r="E57" s="40" t="s">
+      <c r="E57" s="49" t="s">
         <v>241</v>
       </c>
       <c r="F57" s="20" t="s">
@@ -4231,25 +4231,25 @@
       <c r="G57" s="20" t="s">
         <v>243</v>
       </c>
-      <c r="H57" s="40" t="s">
+      <c r="H57" s="49" t="s">
         <v>244</v>
       </c>
-      <c r="I57" s="40" t="s">
+      <c r="I57" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J57" s="40" t="s">
+      <c r="J57" s="49" t="s">
         <v>114</v>
       </c>
-      <c r="K57" s="40" t="s">
+      <c r="K57" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="L57" s="51" t="s">
+      <c r="L57" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M57" s="40" t="s">
+      <c r="M57" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N57" s="40" t="s">
+      <c r="N57" s="49" t="s">
         <v>246</v>
       </c>
       <c r="O57" s="1"/>
@@ -4267,23 +4267,23 @@
     </row>
     <row r="58" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1"/>
-      <c r="B58" s="41"/>
-      <c r="C58" s="41"/>
-      <c r="D58" s="41"/>
-      <c r="E58" s="41"/>
+      <c r="B58" s="51"/>
+      <c r="C58" s="51"/>
+      <c r="D58" s="51"/>
+      <c r="E58" s="51"/>
       <c r="F58" s="20" t="s">
         <v>247</v>
       </c>
       <c r="G58" s="20" t="s">
         <v>248</v>
       </c>
-      <c r="H58" s="41"/>
-      <c r="I58" s="41"/>
-      <c r="J58" s="41"/>
-      <c r="K58" s="41"/>
-      <c r="L58" s="53"/>
-      <c r="M58" s="41"/>
-      <c r="N58" s="41"/>
+      <c r="H58" s="51"/>
+      <c r="I58" s="51"/>
+      <c r="J58" s="51"/>
+      <c r="K58" s="51"/>
+      <c r="L58" s="63"/>
+      <c r="M58" s="51"/>
+      <c r="N58" s="51"/>
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
       <c r="Q58" s="1"/>
@@ -4299,16 +4299,16 @@
     </row>
     <row r="59" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1"/>
-      <c r="B59" s="40" t="s">
+      <c r="B59" s="49" t="s">
         <v>249</v>
       </c>
-      <c r="C59" s="40" t="s">
+      <c r="C59" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="D59" s="40" t="s">
+      <c r="D59" s="49" t="s">
         <v>250</v>
       </c>
-      <c r="E59" s="40" t="s">
+      <c r="E59" s="49" t="s">
         <v>251</v>
       </c>
       <c r="F59" s="20" t="s">
@@ -4317,25 +4317,25 @@
       <c r="G59" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="H59" s="40" t="s">
+      <c r="H59" s="49" t="s">
         <v>254</v>
       </c>
-      <c r="I59" s="40" t="s">
+      <c r="I59" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J59" s="40" t="s">
+      <c r="J59" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="K59" s="40" t="s">
+      <c r="K59" s="49" t="s">
         <v>255</v>
       </c>
-      <c r="L59" s="51" t="s">
+      <c r="L59" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M59" s="40" t="s">
+      <c r="M59" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N59" s="40" t="s">
+      <c r="N59" s="49" t="s">
         <v>256</v>
       </c>
       <c r="O59" s="1"/>
@@ -4353,23 +4353,23 @@
     </row>
     <row r="60" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1"/>
-      <c r="B60" s="41"/>
-      <c r="C60" s="41"/>
-      <c r="D60" s="41"/>
-      <c r="E60" s="41"/>
+      <c r="B60" s="51"/>
+      <c r="C60" s="51"/>
+      <c r="D60" s="51"/>
+      <c r="E60" s="51"/>
       <c r="F60" s="20" t="s">
         <v>257</v>
       </c>
       <c r="G60" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="H60" s="41"/>
-      <c r="I60" s="41"/>
-      <c r="J60" s="41"/>
-      <c r="K60" s="41"/>
-      <c r="L60" s="53"/>
-      <c r="M60" s="41"/>
-      <c r="N60" s="41"/>
+      <c r="H60" s="51"/>
+      <c r="I60" s="51"/>
+      <c r="J60" s="51"/>
+      <c r="K60" s="51"/>
+      <c r="L60" s="63"/>
+      <c r="M60" s="51"/>
+      <c r="N60" s="51"/>
       <c r="O60" s="1"/>
       <c r="P60" s="1"/>
       <c r="Q60" s="1"/>
@@ -4385,16 +4385,16 @@
     </row>
     <row r="61" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1"/>
-      <c r="B61" s="40" t="s">
+      <c r="B61" s="49" t="s">
         <v>259</v>
       </c>
-      <c r="C61" s="40" t="s">
+      <c r="C61" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="D61" s="40" t="s">
+      <c r="D61" s="49" t="s">
         <v>261</v>
       </c>
-      <c r="E61" s="40" t="s">
+      <c r="E61" s="49" t="s">
         <v>262</v>
       </c>
       <c r="F61" s="20" t="s">
@@ -4403,25 +4403,25 @@
       <c r="G61" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="H61" s="40" t="s">
+      <c r="H61" s="49" t="s">
         <v>265</v>
       </c>
-      <c r="I61" s="40" t="s">
+      <c r="I61" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J61" s="40" t="s">
+      <c r="J61" s="49" t="s">
         <v>234</v>
       </c>
-      <c r="K61" s="40" t="s">
+      <c r="K61" s="49" t="s">
         <v>266</v>
       </c>
-      <c r="L61" s="51" t="s">
+      <c r="L61" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M61" s="40" t="s">
+      <c r="M61" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N61" s="40" t="s">
+      <c r="N61" s="49" t="s">
         <v>267</v>
       </c>
       <c r="O61" s="1"/>
@@ -4439,23 +4439,23 @@
     </row>
     <row r="62" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1"/>
-      <c r="B62" s="42"/>
-      <c r="C62" s="42"/>
-      <c r="D62" s="42"/>
-      <c r="E62" s="42"/>
+      <c r="B62" s="50"/>
+      <c r="C62" s="50"/>
+      <c r="D62" s="50"/>
+      <c r="E62" s="50"/>
       <c r="F62" s="20" t="s">
         <v>268</v>
       </c>
       <c r="G62" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="H62" s="42"/>
-      <c r="I62" s="42"/>
-      <c r="J62" s="42"/>
-      <c r="K62" s="42"/>
-      <c r="L62" s="52"/>
-      <c r="M62" s="42"/>
-      <c r="N62" s="42"/>
+      <c r="H62" s="50"/>
+      <c r="I62" s="50"/>
+      <c r="J62" s="50"/>
+      <c r="K62" s="50"/>
+      <c r="L62" s="62"/>
+      <c r="M62" s="50"/>
+      <c r="N62" s="50"/>
       <c r="O62" s="1"/>
       <c r="P62" s="1"/>
       <c r="Q62" s="1"/>
@@ -4471,23 +4471,23 @@
     </row>
     <row r="63" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1"/>
-      <c r="B63" s="41"/>
-      <c r="C63" s="41"/>
-      <c r="D63" s="41"/>
-      <c r="E63" s="41"/>
+      <c r="B63" s="51"/>
+      <c r="C63" s="51"/>
+      <c r="D63" s="51"/>
+      <c r="E63" s="51"/>
       <c r="F63" s="20" t="s">
         <v>270</v>
       </c>
       <c r="G63" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="H63" s="41"/>
-      <c r="I63" s="41"/>
-      <c r="J63" s="41"/>
-      <c r="K63" s="41"/>
-      <c r="L63" s="53"/>
-      <c r="M63" s="41"/>
-      <c r="N63" s="41"/>
+      <c r="H63" s="51"/>
+      <c r="I63" s="51"/>
+      <c r="J63" s="51"/>
+      <c r="K63" s="51"/>
+      <c r="L63" s="63"/>
+      <c r="M63" s="51"/>
+      <c r="N63" s="51"/>
       <c r="O63" s="1"/>
       <c r="P63" s="1"/>
       <c r="Q63" s="1"/>
@@ -4503,16 +4503,16 @@
     </row>
     <row r="64" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1"/>
-      <c r="B64" s="40" t="s">
+      <c r="B64" s="49" t="s">
         <v>272</v>
       </c>
-      <c r="C64" s="40" t="s">
+      <c r="C64" s="49" t="s">
         <v>273</v>
       </c>
-      <c r="D64" s="40" t="s">
+      <c r="D64" s="49" t="s">
         <v>274</v>
       </c>
-      <c r="E64" s="40" t="s">
+      <c r="E64" s="49" t="s">
         <v>275</v>
       </c>
       <c r="F64" s="20" t="s">
@@ -4521,25 +4521,25 @@
       <c r="G64" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H64" s="40" t="s">
+      <c r="H64" s="49" t="s">
         <v>278</v>
       </c>
-      <c r="I64" s="40" t="s">
+      <c r="I64" s="49" t="s">
         <v>279</v>
       </c>
-      <c r="J64" s="40" t="s">
+      <c r="J64" s="49" t="s">
         <v>280</v>
       </c>
-      <c r="K64" s="40" t="s">
+      <c r="K64" s="49" t="s">
         <v>281</v>
       </c>
-      <c r="L64" s="51" t="s">
+      <c r="L64" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M64" s="40" t="s">
+      <c r="M64" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N64" s="40" t="s">
+      <c r="N64" s="49" t="s">
         <v>282</v>
       </c>
       <c r="O64" s="1"/>
@@ -4557,23 +4557,23 @@
     </row>
     <row r="65" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1"/>
-      <c r="B65" s="41"/>
-      <c r="C65" s="41"/>
-      <c r="D65" s="41"/>
-      <c r="E65" s="41"/>
+      <c r="B65" s="51"/>
+      <c r="C65" s="51"/>
+      <c r="D65" s="51"/>
+      <c r="E65" s="51"/>
       <c r="F65" s="20" t="s">
         <v>283</v>
       </c>
       <c r="G65" s="20" t="s">
         <v>284</v>
       </c>
-      <c r="H65" s="41"/>
-      <c r="I65" s="41"/>
-      <c r="J65" s="41"/>
-      <c r="K65" s="41"/>
-      <c r="L65" s="53"/>
-      <c r="M65" s="41"/>
-      <c r="N65" s="41"/>
+      <c r="H65" s="51"/>
+      <c r="I65" s="51"/>
+      <c r="J65" s="51"/>
+      <c r="K65" s="51"/>
+      <c r="L65" s="63"/>
+      <c r="M65" s="51"/>
+      <c r="N65" s="51"/>
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
       <c r="Q65" s="1"/>
@@ -4589,16 +4589,16 @@
     </row>
     <row r="66" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1"/>
-      <c r="B66" s="40" t="s">
+      <c r="B66" s="49" t="s">
         <v>285</v>
       </c>
-      <c r="C66" s="40" t="s">
+      <c r="C66" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="D66" s="40" t="s">
+      <c r="D66" s="49" t="s">
         <v>286</v>
       </c>
-      <c r="E66" s="40" t="s">
+      <c r="E66" s="49" t="s">
         <v>287</v>
       </c>
       <c r="F66" s="20" t="s">
@@ -4607,25 +4607,25 @@
       <c r="G66" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="H66" s="40" t="s">
+      <c r="H66" s="49" t="s">
         <v>290</v>
       </c>
-      <c r="I66" s="40" t="s">
+      <c r="I66" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="J66" s="40" t="s">
+      <c r="J66" s="49" t="s">
         <v>291</v>
       </c>
-      <c r="K66" s="40" t="s">
+      <c r="K66" s="49" t="s">
         <v>292</v>
       </c>
-      <c r="L66" s="51" t="s">
+      <c r="L66" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="M66" s="40" t="s">
+      <c r="M66" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="N66" s="40" t="s">
+      <c r="N66" s="49" t="s">
         <v>293</v>
       </c>
       <c r="O66" s="1"/>
@@ -4643,23 +4643,23 @@
     </row>
     <row r="67" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1"/>
-      <c r="B67" s="42"/>
-      <c r="C67" s="42"/>
-      <c r="D67" s="42"/>
-      <c r="E67" s="42"/>
+      <c r="B67" s="50"/>
+      <c r="C67" s="50"/>
+      <c r="D67" s="50"/>
+      <c r="E67" s="50"/>
       <c r="F67" s="20" t="s">
         <v>294</v>
       </c>
       <c r="G67" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="H67" s="42"/>
-      <c r="I67" s="42"/>
-      <c r="J67" s="42"/>
-      <c r="K67" s="42"/>
-      <c r="L67" s="52"/>
-      <c r="M67" s="42"/>
-      <c r="N67" s="42"/>
+      <c r="H67" s="50"/>
+      <c r="I67" s="50"/>
+      <c r="J67" s="50"/>
+      <c r="K67" s="50"/>
+      <c r="L67" s="62"/>
+      <c r="M67" s="50"/>
+      <c r="N67" s="50"/>
       <c r="O67" s="1"/>
       <c r="P67" s="1"/>
       <c r="Q67" s="1"/>
@@ -4675,23 +4675,23 @@
     </row>
     <row r="68" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1"/>
-      <c r="B68" s="42"/>
-      <c r="C68" s="42"/>
-      <c r="D68" s="42"/>
-      <c r="E68" s="42"/>
+      <c r="B68" s="50"/>
+      <c r="C68" s="50"/>
+      <c r="D68" s="50"/>
+      <c r="E68" s="50"/>
       <c r="F68" s="20" t="s">
         <v>296</v>
       </c>
       <c r="G68" s="20" t="s">
         <v>297</v>
       </c>
-      <c r="H68" s="42"/>
-      <c r="I68" s="42"/>
-      <c r="J68" s="42"/>
-      <c r="K68" s="42"/>
-      <c r="L68" s="52"/>
-      <c r="M68" s="42"/>
-      <c r="N68" s="42"/>
+      <c r="H68" s="50"/>
+      <c r="I68" s="50"/>
+      <c r="J68" s="50"/>
+      <c r="K68" s="50"/>
+      <c r="L68" s="62"/>
+      <c r="M68" s="50"/>
+      <c r="N68" s="50"/>
       <c r="O68" s="1"/>
       <c r="P68" s="1"/>
       <c r="Q68" s="1"/>
@@ -4707,23 +4707,23 @@
     </row>
     <row r="69" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1"/>
-      <c r="B69" s="41"/>
-      <c r="C69" s="41"/>
-      <c r="D69" s="41"/>
-      <c r="E69" s="41"/>
+      <c r="B69" s="51"/>
+      <c r="C69" s="51"/>
+      <c r="D69" s="51"/>
+      <c r="E69" s="51"/>
       <c r="F69" s="20" t="s">
         <v>298</v>
       </c>
       <c r="G69" s="20" t="s">
         <v>299</v>
       </c>
-      <c r="H69" s="41"/>
-      <c r="I69" s="41"/>
-      <c r="J69" s="41"/>
-      <c r="K69" s="41"/>
-      <c r="L69" s="53"/>
-      <c r="M69" s="41"/>
-      <c r="N69" s="41"/>
+      <c r="H69" s="51"/>
+      <c r="I69" s="51"/>
+      <c r="J69" s="51"/>
+      <c r="K69" s="51"/>
+      <c r="L69" s="63"/>
+      <c r="M69" s="51"/>
+      <c r="N69" s="51"/>
       <c r="O69" s="1"/>
       <c r="P69" s="1"/>
       <c r="Q69" s="1"/>
@@ -31927,6 +31927,226 @@
     </row>
   </sheetData>
   <mergeCells count="238">
+    <mergeCell ref="K64:K65"/>
+    <mergeCell ref="L64:L65"/>
+    <mergeCell ref="M64:M65"/>
+    <mergeCell ref="N64:N65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="H64:H65"/>
+    <mergeCell ref="I64:I65"/>
+    <mergeCell ref="J64:J65"/>
+    <mergeCell ref="K61:K63"/>
+    <mergeCell ref="L61:L63"/>
+    <mergeCell ref="M61:M63"/>
+    <mergeCell ref="N61:N63"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="D61:D63"/>
+    <mergeCell ref="E61:E63"/>
+    <mergeCell ref="H61:H63"/>
+    <mergeCell ref="I61:I63"/>
+    <mergeCell ref="J61:J63"/>
+    <mergeCell ref="K59:K60"/>
+    <mergeCell ref="L59:L60"/>
+    <mergeCell ref="M59:M60"/>
+    <mergeCell ref="N59:N60"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="D59:D60"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="H59:H60"/>
+    <mergeCell ref="I59:I60"/>
+    <mergeCell ref="J59:J60"/>
+    <mergeCell ref="K57:K58"/>
+    <mergeCell ref="L57:L58"/>
+    <mergeCell ref="M57:M58"/>
+    <mergeCell ref="N57:N58"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="D57:D58"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="H57:H58"/>
+    <mergeCell ref="I57:I58"/>
+    <mergeCell ref="J57:J58"/>
+    <mergeCell ref="K55:K56"/>
+    <mergeCell ref="L55:L56"/>
+    <mergeCell ref="M55:M56"/>
+    <mergeCell ref="N55:N56"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="H55:H56"/>
+    <mergeCell ref="I55:I56"/>
+    <mergeCell ref="J55:J56"/>
+    <mergeCell ref="K52:K54"/>
+    <mergeCell ref="L52:L54"/>
+    <mergeCell ref="M52:M54"/>
+    <mergeCell ref="N52:N54"/>
+    <mergeCell ref="B52:B54"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="D52:D54"/>
+    <mergeCell ref="E52:E54"/>
+    <mergeCell ref="H52:H54"/>
+    <mergeCell ref="I52:I54"/>
+    <mergeCell ref="J52:J54"/>
+    <mergeCell ref="K50:K51"/>
+    <mergeCell ref="L50:L51"/>
+    <mergeCell ref="M50:M51"/>
+    <mergeCell ref="N50:N51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="H50:H51"/>
+    <mergeCell ref="I50:I51"/>
+    <mergeCell ref="J50:J51"/>
+    <mergeCell ref="K66:K69"/>
+    <mergeCell ref="L66:L69"/>
+    <mergeCell ref="M66:M69"/>
+    <mergeCell ref="N66:N69"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="I66:I69"/>
+    <mergeCell ref="J66:J69"/>
+    <mergeCell ref="K24:K27"/>
+    <mergeCell ref="L24:L27"/>
+    <mergeCell ref="M24:M27"/>
+    <mergeCell ref="N24:N27"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="C24:C27"/>
+    <mergeCell ref="D24:D27"/>
+    <mergeCell ref="E24:E27"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="I24:I27"/>
+    <mergeCell ref="J24:J27"/>
+    <mergeCell ref="K20:K23"/>
+    <mergeCell ref="L20:L23"/>
+    <mergeCell ref="M20:M23"/>
+    <mergeCell ref="N20:N23"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="D20:D23"/>
+    <mergeCell ref="E20:E23"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="I20:I23"/>
+    <mergeCell ref="J20:J23"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="N16:N19"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="D16:D19"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="I16:I19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="K34:K37"/>
+    <mergeCell ref="L34:L37"/>
+    <mergeCell ref="M34:M37"/>
+    <mergeCell ref="N34:N37"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="I34:I37"/>
+    <mergeCell ref="J34:J37"/>
+    <mergeCell ref="K47:K49"/>
+    <mergeCell ref="L47:L49"/>
+    <mergeCell ref="M47:M49"/>
+    <mergeCell ref="N47:N49"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="D47:D49"/>
+    <mergeCell ref="E47:E49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="I47:I49"/>
+    <mergeCell ref="J47:J49"/>
+    <mergeCell ref="K44:K46"/>
+    <mergeCell ref="L44:L46"/>
+    <mergeCell ref="M44:M46"/>
+    <mergeCell ref="N44:N46"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="D44:D46"/>
+    <mergeCell ref="E44:E46"/>
+    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="I44:I46"/>
+    <mergeCell ref="J44:J46"/>
+    <mergeCell ref="K41:K43"/>
+    <mergeCell ref="L41:L43"/>
+    <mergeCell ref="M41:M43"/>
+    <mergeCell ref="N41:N43"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="D41:D43"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="I41:I43"/>
+    <mergeCell ref="J41:J43"/>
+    <mergeCell ref="K38:K40"/>
+    <mergeCell ref="L38:L40"/>
+    <mergeCell ref="M38:M40"/>
+    <mergeCell ref="N38:N40"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="D38:D40"/>
+    <mergeCell ref="E38:E40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="I38:I40"/>
+    <mergeCell ref="J38:J40"/>
+    <mergeCell ref="K31:K33"/>
+    <mergeCell ref="L31:L33"/>
+    <mergeCell ref="M31:M33"/>
+    <mergeCell ref="N31:N33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="H31:H33"/>
+    <mergeCell ref="I31:I33"/>
+    <mergeCell ref="J31:J33"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="M28:M30"/>
+    <mergeCell ref="N28:N30"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="H28:H30"/>
+    <mergeCell ref="I28:I30"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="K13:K15"/>
+    <mergeCell ref="L13:L15"/>
+    <mergeCell ref="M13:M15"/>
+    <mergeCell ref="N13:N15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="B3:C3"/>
@@ -31945,228 +32165,8 @@
     <mergeCell ref="H7:H10"/>
     <mergeCell ref="I7:I10"/>
     <mergeCell ref="J7:J10"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K13:K15"/>
-    <mergeCell ref="L13:L15"/>
-    <mergeCell ref="M13:M15"/>
-    <mergeCell ref="N13:N15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="H13:H15"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="J13:J15"/>
-    <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="M28:M30"/>
-    <mergeCell ref="N28:N30"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="H28:H30"/>
-    <mergeCell ref="I28:I30"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="K31:K33"/>
-    <mergeCell ref="L31:L33"/>
-    <mergeCell ref="M31:M33"/>
-    <mergeCell ref="N31:N33"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="H31:H33"/>
-    <mergeCell ref="I31:I33"/>
-    <mergeCell ref="J31:J33"/>
-    <mergeCell ref="K38:K40"/>
-    <mergeCell ref="L38:L40"/>
-    <mergeCell ref="M38:M40"/>
-    <mergeCell ref="N38:N40"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="D38:D40"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="H38:H40"/>
-    <mergeCell ref="I38:I40"/>
-    <mergeCell ref="J38:J40"/>
-    <mergeCell ref="K41:K43"/>
-    <mergeCell ref="L41:L43"/>
-    <mergeCell ref="M41:M43"/>
-    <mergeCell ref="N41:N43"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="D41:D43"/>
-    <mergeCell ref="E41:E43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="I41:I43"/>
-    <mergeCell ref="J41:J43"/>
-    <mergeCell ref="K44:K46"/>
-    <mergeCell ref="L44:L46"/>
-    <mergeCell ref="M44:M46"/>
-    <mergeCell ref="N44:N46"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="D44:D46"/>
-    <mergeCell ref="E44:E46"/>
-    <mergeCell ref="H44:H46"/>
-    <mergeCell ref="I44:I46"/>
-    <mergeCell ref="J44:J46"/>
-    <mergeCell ref="K47:K49"/>
-    <mergeCell ref="L47:L49"/>
-    <mergeCell ref="M47:M49"/>
-    <mergeCell ref="N47:N49"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="D47:D49"/>
-    <mergeCell ref="E47:E49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="I47:I49"/>
-    <mergeCell ref="J47:J49"/>
-    <mergeCell ref="K34:K37"/>
-    <mergeCell ref="L34:L37"/>
-    <mergeCell ref="M34:M37"/>
-    <mergeCell ref="N34:N37"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="I34:I37"/>
-    <mergeCell ref="J34:J37"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="N16:N19"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="D16:D19"/>
-    <mergeCell ref="E16:E19"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="I16:I19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="K20:K23"/>
-    <mergeCell ref="L20:L23"/>
-    <mergeCell ref="M20:M23"/>
-    <mergeCell ref="N20:N23"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="D20:D23"/>
-    <mergeCell ref="E20:E23"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="I20:I23"/>
-    <mergeCell ref="J20:J23"/>
-    <mergeCell ref="K24:K27"/>
-    <mergeCell ref="L24:L27"/>
-    <mergeCell ref="M24:M27"/>
-    <mergeCell ref="N24:N27"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="C24:C27"/>
-    <mergeCell ref="D24:D27"/>
-    <mergeCell ref="E24:E27"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="I24:I27"/>
-    <mergeCell ref="J24:J27"/>
-    <mergeCell ref="K66:K69"/>
-    <mergeCell ref="L66:L69"/>
-    <mergeCell ref="M66:M69"/>
-    <mergeCell ref="N66:N69"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="I66:I69"/>
-    <mergeCell ref="J66:J69"/>
-    <mergeCell ref="K50:K51"/>
-    <mergeCell ref="L50:L51"/>
-    <mergeCell ref="M50:M51"/>
-    <mergeCell ref="N50:N51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="H50:H51"/>
-    <mergeCell ref="I50:I51"/>
-    <mergeCell ref="J50:J51"/>
-    <mergeCell ref="K52:K54"/>
-    <mergeCell ref="L52:L54"/>
-    <mergeCell ref="M52:M54"/>
-    <mergeCell ref="N52:N54"/>
-    <mergeCell ref="B52:B54"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="D52:D54"/>
-    <mergeCell ref="E52:E54"/>
-    <mergeCell ref="H52:H54"/>
-    <mergeCell ref="I52:I54"/>
-    <mergeCell ref="J52:J54"/>
-    <mergeCell ref="K55:K56"/>
-    <mergeCell ref="L55:L56"/>
-    <mergeCell ref="M55:M56"/>
-    <mergeCell ref="N55:N56"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="H55:H56"/>
-    <mergeCell ref="I55:I56"/>
-    <mergeCell ref="J55:J56"/>
-    <mergeCell ref="K57:K58"/>
-    <mergeCell ref="L57:L58"/>
-    <mergeCell ref="M57:M58"/>
-    <mergeCell ref="N57:N58"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="D57:D58"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="H57:H58"/>
-    <mergeCell ref="I57:I58"/>
-    <mergeCell ref="J57:J58"/>
-    <mergeCell ref="K59:K60"/>
-    <mergeCell ref="L59:L60"/>
-    <mergeCell ref="M59:M60"/>
-    <mergeCell ref="N59:N60"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="D59:D60"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="H59:H60"/>
-    <mergeCell ref="I59:I60"/>
-    <mergeCell ref="J59:J60"/>
-    <mergeCell ref="K61:K63"/>
-    <mergeCell ref="L61:L63"/>
-    <mergeCell ref="M61:M63"/>
-    <mergeCell ref="N61:N63"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="D61:D63"/>
-    <mergeCell ref="E61:E63"/>
-    <mergeCell ref="H61:H63"/>
-    <mergeCell ref="I61:I63"/>
-    <mergeCell ref="J61:J63"/>
-    <mergeCell ref="K64:K65"/>
-    <mergeCell ref="L64:L65"/>
-    <mergeCell ref="M64:M65"/>
-    <mergeCell ref="N64:N65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="H64:H65"/>
-    <mergeCell ref="I64:I65"/>
-    <mergeCell ref="J64:J65"/>
   </mergeCells>
-  <conditionalFormatting sqref="B7:F1040 G11:H1040 I7:N1040">
+  <conditionalFormatting sqref="B7:F1040 I7:N1040 G11:H1040">
     <cfRule type="expression" dxfId="24" priority="1" stopIfTrue="1">
       <formula>$M7="En Progreso"</formula>
     </cfRule>
@@ -32396,7 +32396,7 @@
       <c r="G6" s="33" t="s">
         <v>305</v>
       </c>
-      <c r="H6" s="63">
+      <c r="H6" s="40">
         <v>46207</v>
       </c>
       <c r="I6" s="35" t="s">
@@ -35590,30 +35590,30 @@
       <c r="H998" s="13"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H3:I15 B3:F15">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="B3:F15 H3:I15">
+    <cfRule type="expression" dxfId="6" priority="1" stopIfTrue="1">
       <formula>OR($G3="Planned",$G3="Unplanned")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="2" stopIfTrue="1">
       <formula>$G3="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F16">
-    <cfRule type="expression" dxfId="6" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
       <formula>$G16="Planned"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
       <formula>$G16="Ongoing"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G15">
-    <cfRule type="expression" dxfId="4" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
       <formula>$G3="Planned"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
       <formula>$G3="Ongoing"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="7" stopIfTrue="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="7" stopIfTrue="1" operator="equal">
       <formula>"Unplanned"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
documentos de finalizacion de sprint 1
</commit_message>
<xml_diff>
--- a/docs/Planificación/01 Backlog Detallado del Producto.xlsx
+++ b/docs/Planificación/01 Backlog Detallado del Producto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Periodo Final 2026-10\Taller de Proyectos 2\semana 1\Planner\Taller_Proyectos_2\docs\Planificación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4AF4C0-C800-4F54-A558-972CBE570AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A905D38-2A1C-4D51-B2C7-39FE164DE893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog del Producto" sheetId="1" r:id="rId1"/>
@@ -1453,7 +1453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1606,6 +1606,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2031,10 +2034,10 @@
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" customWidth="1"/>
+    <col min="4" max="4" width="59.7109375" customWidth="1"/>
+    <col min="5" max="5" width="48.42578125" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" customWidth="1"/>
-    <col min="7" max="7" width="56.28515625" customWidth="1"/>
+    <col min="7" max="7" width="88" customWidth="1"/>
     <col min="8" max="8" width="53.140625" customWidth="1"/>
     <col min="9" max="9" width="10.28515625" customWidth="1"/>
     <col min="10" max="11" width="15" customWidth="1"/>
@@ -2265,41 +2268,41 @@
     </row>
     <row r="7" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="49" t="s">
+      <c r="C7" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="D7" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E7" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="49" t="s">
+      <c r="H7" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="49" t="s">
+      <c r="I7" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="J7" s="49" t="s">
+      <c r="J7" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="49"/>
+      <c r="K7" s="52"/>
       <c r="L7" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="M7" s="49" t="s">
+      <c r="M7" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="N7" s="49" t="s">
+      <c r="N7" s="52" t="s">
         <v>34</v>
       </c>
       <c r="O7" s="1"/>
@@ -2317,23 +2320,23 @@
     </row>
     <row r="8" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
-      <c r="B8" s="50"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="50"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="20" t="s">
+      <c r="B8" s="53"/>
+      <c r="C8" s="53"/>
+      <c r="D8" s="53"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="50"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="50"/>
-      <c r="K8" s="50"/>
+      <c r="H8" s="53"/>
+      <c r="I8" s="53"/>
+      <c r="J8" s="53"/>
+      <c r="K8" s="53"/>
       <c r="L8" s="53"/>
-      <c r="M8" s="50"/>
-      <c r="N8" s="50"/>
+      <c r="M8" s="53"/>
+      <c r="N8" s="53"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
@@ -2349,23 +2352,23 @@
     </row>
     <row r="9" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="20" t="s">
+      <c r="B9" s="53"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="53"/>
+      <c r="E9" s="53"/>
+      <c r="F9" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="50"/>
+      <c r="H9" s="53"/>
+      <c r="I9" s="53"/>
+      <c r="J9" s="53"/>
+      <c r="K9" s="53"/>
       <c r="L9" s="53"/>
-      <c r="M9" s="50"/>
-      <c r="N9" s="50"/>
+      <c r="M9" s="53"/>
+      <c r="N9" s="53"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
@@ -2381,23 +2384,23 @@
     </row>
     <row r="10" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
-      <c r="B10" s="51"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="20" t="s">
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="51"/>
-      <c r="I10" s="51"/>
-      <c r="J10" s="51"/>
-      <c r="K10" s="51"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
+      <c r="J10" s="54"/>
+      <c r="K10" s="54"/>
       <c r="L10" s="54"/>
-      <c r="M10" s="51"/>
-      <c r="N10" s="51"/>
+      <c r="M10" s="54"/>
+      <c r="N10" s="54"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
@@ -2413,43 +2416,43 @@
     </row>
     <row r="11" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="49" t="s">
+      <c r="B11" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="49" t="s">
+      <c r="C11" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="49" t="s">
+      <c r="D11" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="49" t="s">
+      <c r="E11" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="F11" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="64" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="49" t="s">
+      <c r="H11" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="49" t="s">
+      <c r="I11" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="J11" s="49" t="s">
+      <c r="J11" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="K11" s="49" t="s">
+      <c r="K11" s="52" t="s">
         <v>49</v>
       </c>
       <c r="L11" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="M11" s="49" t="s">
+      <c r="M11" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="N11" s="49" t="s">
+      <c r="N11" s="52" t="s">
         <v>50</v>
       </c>
       <c r="O11" s="1"/>
@@ -2467,23 +2470,23 @@
     </row>
     <row r="12" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="51"/>
-      <c r="C12" s="51"/>
-      <c r="D12" s="51"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="20" t="s">
+      <c r="B12" s="54"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="51"/>
-      <c r="I12" s="51"/>
-      <c r="J12" s="51"/>
-      <c r="K12" s="51"/>
+      <c r="H12" s="54"/>
+      <c r="I12" s="54"/>
+      <c r="J12" s="54"/>
+      <c r="K12" s="54"/>
       <c r="L12" s="54"/>
-      <c r="M12" s="51"/>
-      <c r="N12" s="51"/>
+      <c r="M12" s="54"/>
+      <c r="N12" s="54"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
@@ -2499,43 +2502,43 @@
     </row>
     <row r="13" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="49" t="s">
+      <c r="B13" s="52" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="49" t="s">
+      <c r="D13" s="52" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="49" t="s">
+      <c r="E13" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="F13" s="64" t="s">
         <v>56</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="64" t="s">
         <v>57</v>
       </c>
-      <c r="H13" s="49" t="s">
+      <c r="H13" s="52" t="s">
         <v>58</v>
       </c>
-      <c r="I13" s="49" t="s">
+      <c r="I13" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="J13" s="49" t="s">
+      <c r="J13" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="K13" s="49" t="s">
+      <c r="K13" s="52" t="s">
         <v>59</v>
       </c>
       <c r="L13" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="M13" s="49" t="s">
+      <c r="M13" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="N13" s="49" t="s">
+      <c r="N13" s="52" t="s">
         <v>60</v>
       </c>
       <c r="O13" s="1"/>
@@ -2553,23 +2556,23 @@
     </row>
     <row r="14" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="50"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="20" t="s">
+      <c r="B14" s="53"/>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="G14" s="64" t="s">
         <v>62</v>
       </c>
-      <c r="H14" s="50"/>
-      <c r="I14" s="50"/>
-      <c r="J14" s="50"/>
-      <c r="K14" s="50"/>
+      <c r="H14" s="53"/>
+      <c r="I14" s="53"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="53"/>
       <c r="L14" s="53"/>
-      <c r="M14" s="50"/>
-      <c r="N14" s="50"/>
+      <c r="M14" s="53"/>
+      <c r="N14" s="53"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
@@ -2585,23 +2588,23 @@
     </row>
     <row r="15" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="51"/>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
-      <c r="E15" s="51"/>
-      <c r="F15" s="20" t="s">
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="51"/>
-      <c r="I15" s="51"/>
-      <c r="J15" s="51"/>
-      <c r="K15" s="51"/>
+      <c r="H15" s="54"/>
+      <c r="I15" s="54"/>
+      <c r="J15" s="54"/>
+      <c r="K15" s="54"/>
       <c r="L15" s="54"/>
-      <c r="M15" s="51"/>
-      <c r="N15" s="51"/>
+      <c r="M15" s="54"/>
+      <c r="N15" s="54"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
@@ -32304,14 +32307,14 @@
         <v>19</v>
       </c>
       <c r="E3" s="32">
-        <f t="shared" ref="E3:E6" si="0">IF(AND(C3&lt;&gt;"",D3&lt;&gt;""),C3+D3-1,"")</f>
+        <f t="shared" ref="E3:E5" si="0">IF(AND(C3&lt;&gt;"",D3&lt;&gt;""),C3+D3-1,"")</f>
         <v>46143</v>
       </c>
       <c r="F3" s="29">
         <v>18</v>
       </c>
       <c r="G3" s="33" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H3" s="34">
         <v>46145</v>
@@ -35591,7 +35594,7 @@
       <c r="H998" s="13"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H3:I15 B3:F15">
+  <conditionalFormatting sqref="B3:F15 H3:I15">
     <cfRule type="expression" dxfId="6" priority="1" stopIfTrue="1">
       <formula>OR($G3="Planned",$G3="Unplanned")</formula>
     </cfRule>

</xml_diff>

<commit_message>
ajuste de fecha sprint 1 y sprint 2 - planificacion del sprint 2
</commit_message>
<xml_diff>
--- a/docs/Planificación/01 Backlog Detallado del Producto.xlsx
+++ b/docs/Planificación/01 Backlog Detallado del Producto.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Periodo Final 2026-10\Taller de Proyectos 2\semana 1\Planner\Taller_Proyectos_2\docs\Planificación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\Periodo Final 2026-10\Taller de Proyectos 2\semana 1\Planner\Taller_Proyectos_2\docs\Planificación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A905D38-2A1C-4D51-B2C7-39FE164DE893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="330" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog del Producto" sheetId="1" r:id="rId1"/>
@@ -46,7 +45,7 @@
     <definedName name="TrendOffset">#REF!</definedName>
     <definedName name="TrendSprintCount">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="iiWbymOwducJ8ZzFrdiwAJ0giCg4NOprm4hI8W6yQk4="/>
@@ -56,12 +55,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="B6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -78,7 +77,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="F6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -95,7 +94,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="I6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -113,7 +112,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="J6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -132,7 +131,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="K6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -149,7 +148,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="L6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -168,7 +167,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="M6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1188,10 +1187,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -1453,7 +1451,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1546,7 +1544,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1563,6 +1561,34 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1581,32 +1607,7 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1816,6 +1817,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF99FF66"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2024,7 +2030,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2082,14 +2088,14 @@
     </row>
     <row r="2" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="43" t="s">
+      <c r="C2" s="58"/>
+      <c r="D2" s="59" t="s">
         <v>312</v>
       </c>
-      <c r="E2" s="44"/>
+      <c r="E2" s="60"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="7"/>
@@ -2116,14 +2122,14 @@
     </row>
     <row r="3" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="43" t="s">
+      <c r="C3" s="58"/>
+      <c r="D3" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="44"/>
+      <c r="E3" s="60"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="7"/>
@@ -2180,25 +2186,25 @@
     </row>
     <row r="5" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="47" t="s">
+      <c r="C5" s="62"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="44"/>
-      <c r="H5" s="48" t="s">
+      <c r="G5" s="60"/>
+      <c r="H5" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="46"/>
-      <c r="J5" s="46"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="46"/>
-      <c r="M5" s="46"/>
-      <c r="N5" s="44"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="62"/>
+      <c r="L5" s="62"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="60"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
@@ -2268,41 +2274,41 @@
     </row>
     <row r="7" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
-      <c r="B7" s="52" t="s">
+      <c r="B7" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="52" t="s">
+      <c r="D7" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="52" t="s">
+      <c r="E7" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="64" t="s">
+      <c r="F7" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="64" t="s">
+      <c r="G7" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="52" t="s">
+      <c r="H7" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="52" t="s">
+      <c r="I7" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="J7" s="52" t="s">
+      <c r="J7" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="52"/>
-      <c r="L7" s="52" t="s">
+      <c r="K7" s="54"/>
+      <c r="L7" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="M7" s="52" t="s">
-        <v>1</v>
-      </c>
-      <c r="N7" s="52" t="s">
+      <c r="M7" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="N7" s="54" t="s">
         <v>34</v>
       </c>
       <c r="O7" s="1"/>
@@ -2320,23 +2326,23 @@
     </row>
     <row r="8" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
-      <c r="B8" s="53"/>
-      <c r="C8" s="53"/>
-      <c r="D8" s="53"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="64" t="s">
+      <c r="B8" s="55"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="64" t="s">
+      <c r="G8" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="53"/>
-      <c r="K8" s="53"/>
-      <c r="L8" s="53"/>
-      <c r="M8" s="53"/>
-      <c r="N8" s="53"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="55"/>
+      <c r="L8" s="55"/>
+      <c r="M8" s="55"/>
+      <c r="N8" s="55"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
@@ -2352,23 +2358,23 @@
     </row>
     <row r="9" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="53"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="64" t="s">
+      <c r="B9" s="55"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="64" t="s">
+      <c r="G9" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="53"/>
-      <c r="I9" s="53"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
-      <c r="M9" s="53"/>
-      <c r="N9" s="53"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="55"/>
+      <c r="M9" s="55"/>
+      <c r="N9" s="55"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
@@ -2384,23 +2390,23 @@
     </row>
     <row r="10" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="64" t="s">
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="64" t="s">
+      <c r="G10" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
-      <c r="J10" s="54"/>
-      <c r="K10" s="54"/>
-      <c r="L10" s="54"/>
-      <c r="M10" s="54"/>
-      <c r="N10" s="54"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="56"/>
+      <c r="L10" s="56"/>
+      <c r="M10" s="56"/>
+      <c r="N10" s="56"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
@@ -2416,43 +2422,43 @@
     </row>
     <row r="11" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="52" t="s">
+      <c r="B11" s="54" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="C11" s="54" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="52" t="s">
+      <c r="E11" s="54" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="64" t="s">
+      <c r="F11" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="64" t="s">
+      <c r="G11" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="52" t="s">
+      <c r="H11" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="52" t="s">
+      <c r="I11" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="J11" s="52" t="s">
+      <c r="J11" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="K11" s="52" t="s">
+      <c r="K11" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="52" t="s">
+      <c r="L11" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="M11" s="52" t="s">
-        <v>1</v>
-      </c>
-      <c r="N11" s="52" t="s">
+      <c r="M11" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="N11" s="54" t="s">
         <v>50</v>
       </c>
       <c r="O11" s="1"/>
@@ -2470,23 +2476,23 @@
     </row>
     <row r="12" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="54"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="64" t="s">
+      <c r="B12" s="56"/>
+      <c r="C12" s="56"/>
+      <c r="D12" s="56"/>
+      <c r="E12" s="56"/>
+      <c r="F12" s="41" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="64" t="s">
+      <c r="G12" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="54"/>
-      <c r="I12" s="54"/>
-      <c r="J12" s="54"/>
-      <c r="K12" s="54"/>
-      <c r="L12" s="54"/>
-      <c r="M12" s="54"/>
-      <c r="N12" s="54"/>
+      <c r="H12" s="56"/>
+      <c r="I12" s="56"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="56"/>
+      <c r="L12" s="56"/>
+      <c r="M12" s="56"/>
+      <c r="N12" s="56"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
@@ -2502,43 +2508,43 @@
     </row>
     <row r="13" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="52" t="s">
+      <c r="B13" s="54" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="52" t="s">
+      <c r="C13" s="54" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="52" t="s">
+      <c r="D13" s="54" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="52" t="s">
+      <c r="E13" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="64" t="s">
+      <c r="F13" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="G13" s="64" t="s">
+      <c r="G13" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="H13" s="52" t="s">
+      <c r="H13" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="I13" s="52" t="s">
+      <c r="I13" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="J13" s="52" t="s">
+      <c r="J13" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="K13" s="52" t="s">
+      <c r="K13" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="L13" s="52" t="s">
+      <c r="L13" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="M13" s="52" t="s">
-        <v>1</v>
-      </c>
-      <c r="N13" s="52" t="s">
+      <c r="M13" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="N13" s="54" t="s">
         <v>60</v>
       </c>
       <c r="O13" s="1"/>
@@ -2556,23 +2562,23 @@
     </row>
     <row r="14" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="53"/>
-      <c r="C14" s="53"/>
-      <c r="D14" s="53"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="64" t="s">
+      <c r="B14" s="55"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="G14" s="64" t="s">
+      <c r="G14" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="H14" s="53"/>
-      <c r="I14" s="53"/>
-      <c r="J14" s="53"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="53"/>
-      <c r="M14" s="53"/>
-      <c r="N14" s="53"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="55"/>
+      <c r="M14" s="55"/>
+      <c r="N14" s="55"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
@@ -2588,23 +2594,23 @@
     </row>
     <row r="15" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="64" t="s">
+      <c r="B15" s="56"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="41" t="s">
         <v>63</v>
       </c>
-      <c r="G15" s="64" t="s">
+      <c r="G15" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="54"/>
-      <c r="K15" s="54"/>
-      <c r="L15" s="54"/>
-      <c r="M15" s="54"/>
-      <c r="N15" s="54"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="56"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="56"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="56"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
@@ -2620,43 +2626,43 @@
     </row>
     <row r="16" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-      <c r="B16" s="49" t="s">
+      <c r="B16" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="49" t="s">
+      <c r="C16" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="49" t="s">
+      <c r="D16" s="48" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="49" t="s">
+      <c r="E16" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="65" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="65" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="49" t="s">
+      <c r="H16" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="I16" s="49" t="s">
+      <c r="I16" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J16" s="49" t="s">
+      <c r="J16" s="48" t="s">
         <v>72</v>
       </c>
-      <c r="K16" s="49" t="s">
+      <c r="K16" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="L16" s="55" t="s">
+      <c r="L16" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="M16" s="49" t="s">
+      <c r="M16" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="N16" s="49"/>
+      <c r="N16" s="48"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
@@ -2672,23 +2678,23 @@
     </row>
     <row r="17" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="50"/>
-      <c r="C17" s="50"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="20" t="s">
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="G17" s="20" t="s">
+      <c r="G17" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="H17" s="50"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="50"/>
-      <c r="K17" s="50"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="50"/>
-      <c r="N17" s="50"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
@@ -2704,23 +2710,23 @@
     </row>
     <row r="18" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="50"/>
-      <c r="C18" s="50"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="20" t="s">
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="65" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="50"/>
-      <c r="K18" s="50"/>
-      <c r="L18" s="56"/>
-      <c r="M18" s="50"/>
-      <c r="N18" s="50"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="49"/>
+      <c r="L18" s="49"/>
+      <c r="M18" s="49"/>
+      <c r="N18" s="49"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
@@ -2736,23 +2742,23 @@
     </row>
     <row r="19" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="51"/>
-      <c r="C19" s="51"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="51"/>
-      <c r="F19" s="20" t="s">
+      <c r="B19" s="50"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="65" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="H19" s="51"/>
-      <c r="I19" s="51"/>
-      <c r="J19" s="51"/>
-      <c r="K19" s="51"/>
-      <c r="L19" s="57"/>
-      <c r="M19" s="51"/>
-      <c r="N19" s="51"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
@@ -2768,43 +2774,43 @@
     </row>
     <row r="20" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="49" t="s">
+      <c r="B20" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="49" t="s">
+      <c r="C20" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="49" t="s">
+      <c r="D20" s="48" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="49" t="s">
+      <c r="E20" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="F20" s="65" t="s">
         <v>83</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="H20" s="49" t="s">
+      <c r="H20" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="I20" s="49" t="s">
+      <c r="I20" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J20" s="49" t="s">
+      <c r="J20" s="48" t="s">
         <v>86</v>
       </c>
-      <c r="K20" s="49" t="s">
+      <c r="K20" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="L20" s="55" t="s">
+      <c r="L20" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="M20" s="49" t="s">
+      <c r="M20" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="N20" s="49" t="s">
+      <c r="N20" s="48" t="s">
         <v>87</v>
       </c>
       <c r="O20" s="1"/>
@@ -2822,23 +2828,23 @@
     </row>
     <row r="21" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="50"/>
-      <c r="C21" s="50"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="20" t="s">
+      <c r="B21" s="49"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="G21" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="50"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="50"/>
-      <c r="K21" s="50"/>
-      <c r="L21" s="56"/>
-      <c r="M21" s="50"/>
-      <c r="N21" s="50"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="49"/>
+      <c r="N21" s="49"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
@@ -2854,23 +2860,23 @@
     </row>
     <row r="22" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="50"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="20" t="s">
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="65" t="s">
         <v>90</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="65" t="s">
         <v>91</v>
       </c>
-      <c r="H22" s="50"/>
-      <c r="I22" s="50"/>
-      <c r="J22" s="50"/>
-      <c r="K22" s="50"/>
-      <c r="L22" s="56"/>
-      <c r="M22" s="50"/>
-      <c r="N22" s="50"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="49"/>
+      <c r="L22" s="49"/>
+      <c r="M22" s="49"/>
+      <c r="N22" s="49"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
@@ -2886,23 +2892,23 @@
     </row>
     <row r="23" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
-      <c r="B23" s="51"/>
-      <c r="C23" s="51"/>
-      <c r="D23" s="51"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="20" t="s">
+      <c r="B23" s="50"/>
+      <c r="C23" s="50"/>
+      <c r="D23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="65" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="20" t="s">
+      <c r="G23" s="65" t="s">
         <v>93</v>
       </c>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
-      <c r="J23" s="51"/>
-      <c r="K23" s="51"/>
-      <c r="L23" s="57"/>
-      <c r="M23" s="51"/>
-      <c r="N23" s="51"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="50"/>
+      <c r="J23" s="50"/>
+      <c r="K23" s="50"/>
+      <c r="L23" s="50"/>
+      <c r="M23" s="50"/>
+      <c r="N23" s="50"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
@@ -2918,43 +2924,43 @@
     </row>
     <row r="24" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
-      <c r="B24" s="49" t="s">
+      <c r="B24" s="48" t="s">
         <v>94</v>
       </c>
-      <c r="C24" s="49" t="s">
+      <c r="C24" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="E24" s="49" t="s">
+      <c r="E24" s="48" t="s">
         <v>96</v>
       </c>
-      <c r="F24" s="20" t="s">
+      <c r="F24" s="65" t="s">
         <v>97</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="65" t="s">
         <v>98</v>
       </c>
-      <c r="H24" s="49" t="s">
+      <c r="H24" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="I24" s="49" t="s">
+      <c r="I24" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J24" s="49" t="s">
+      <c r="J24" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="K24" s="49" t="s">
+      <c r="K24" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="L24" s="55" t="s">
+      <c r="L24" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="M24" s="49" t="s">
+      <c r="M24" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="N24" s="49" t="s">
+      <c r="N24" s="48" t="s">
         <v>101</v>
       </c>
       <c r="O24" s="1"/>
@@ -2972,23 +2978,23 @@
     </row>
     <row r="25" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
-      <c r="B25" s="50"/>
-      <c r="C25" s="50"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="20" t="s">
+      <c r="B25" s="49"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="G25" s="20" t="s">
+      <c r="G25" s="65" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="50"/>
-      <c r="K25" s="50"/>
-      <c r="L25" s="56"/>
-      <c r="M25" s="50"/>
-      <c r="N25" s="50"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="49"/>
+      <c r="K25" s="49"/>
+      <c r="L25" s="49"/>
+      <c r="M25" s="49"/>
+      <c r="N25" s="49"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
@@ -3004,23 +3010,23 @@
     </row>
     <row r="26" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
-      <c r="B26" s="50"/>
-      <c r="C26" s="50"/>
-      <c r="D26" s="50"/>
-      <c r="E26" s="50"/>
-      <c r="F26" s="20" t="s">
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="65" t="s">
         <v>104</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="65" t="s">
         <v>105</v>
       </c>
-      <c r="H26" s="50"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="50"/>
-      <c r="K26" s="50"/>
-      <c r="L26" s="56"/>
-      <c r="M26" s="50"/>
-      <c r="N26" s="50"/>
+      <c r="H26" s="49"/>
+      <c r="I26" s="49"/>
+      <c r="J26" s="49"/>
+      <c r="K26" s="49"/>
+      <c r="L26" s="49"/>
+      <c r="M26" s="49"/>
+      <c r="N26" s="49"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
@@ -3036,23 +3042,23 @@
     </row>
     <row r="27" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="20" t="s">
+      <c r="B27" s="50"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="G27" s="20" t="s">
+      <c r="G27" s="65" t="s">
         <v>107</v>
       </c>
-      <c r="H27" s="51"/>
-      <c r="I27" s="51"/>
-      <c r="J27" s="51"/>
-      <c r="K27" s="51"/>
-      <c r="L27" s="57"/>
-      <c r="M27" s="51"/>
-      <c r="N27" s="51"/>
+      <c r="H27" s="50"/>
+      <c r="I27" s="50"/>
+      <c r="J27" s="50"/>
+      <c r="K27" s="50"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="50"/>
+      <c r="N27" s="50"/>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
@@ -3068,43 +3074,43 @@
     </row>
     <row r="28" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
-      <c r="B28" s="49" t="s">
+      <c r="B28" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="C28" s="49" t="s">
+      <c r="C28" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="D28" s="49" t="s">
+      <c r="D28" s="48" t="s">
         <v>109</v>
       </c>
-      <c r="E28" s="49" t="s">
+      <c r="E28" s="48" t="s">
         <v>110</v>
       </c>
-      <c r="F28" s="20" t="s">
+      <c r="F28" s="65" t="s">
         <v>111</v>
       </c>
-      <c r="G28" s="20" t="s">
+      <c r="G28" s="65" t="s">
         <v>112</v>
       </c>
-      <c r="H28" s="49" t="s">
+      <c r="H28" s="48" t="s">
         <v>113</v>
       </c>
-      <c r="I28" s="49" t="s">
+      <c r="I28" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J28" s="49" t="s">
+      <c r="J28" s="48" t="s">
         <v>114</v>
       </c>
-      <c r="K28" s="49" t="s">
+      <c r="K28" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="L28" s="55" t="s">
+      <c r="L28" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="M28" s="49" t="s">
+      <c r="M28" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="N28" s="49" t="s">
+      <c r="N28" s="48" t="s">
         <v>115</v>
       </c>
       <c r="O28" s="1"/>
@@ -3122,23 +3128,23 @@
     </row>
     <row r="29" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
-      <c r="B29" s="50"/>
-      <c r="C29" s="50"/>
-      <c r="D29" s="50"/>
-      <c r="E29" s="50"/>
-      <c r="F29" s="20" t="s">
+      <c r="B29" s="49"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="65" t="s">
         <v>117</v>
       </c>
-      <c r="H29" s="50"/>
-      <c r="I29" s="50"/>
-      <c r="J29" s="50"/>
-      <c r="K29" s="50"/>
-      <c r="L29" s="56"/>
-      <c r="M29" s="50"/>
-      <c r="N29" s="50"/>
+      <c r="H29" s="49"/>
+      <c r="I29" s="49"/>
+      <c r="J29" s="49"/>
+      <c r="K29" s="49"/>
+      <c r="L29" s="49"/>
+      <c r="M29" s="49"/>
+      <c r="N29" s="49"/>
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
@@ -3154,23 +3160,23 @@
     </row>
     <row r="30" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
-      <c r="B30" s="51"/>
-      <c r="C30" s="51"/>
-      <c r="D30" s="51"/>
-      <c r="E30" s="51"/>
-      <c r="F30" s="20" t="s">
+      <c r="B30" s="50"/>
+      <c r="C30" s="50"/>
+      <c r="D30" s="50"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="65" t="s">
         <v>118</v>
       </c>
-      <c r="G30" s="20" t="s">
+      <c r="G30" s="65" t="s">
         <v>119</v>
       </c>
-      <c r="H30" s="51"/>
-      <c r="I30" s="51"/>
-      <c r="J30" s="51"/>
-      <c r="K30" s="51"/>
-      <c r="L30" s="57"/>
-      <c r="M30" s="51"/>
-      <c r="N30" s="51"/>
+      <c r="H30" s="50"/>
+      <c r="I30" s="50"/>
+      <c r="J30" s="50"/>
+      <c r="K30" s="50"/>
+      <c r="L30" s="50"/>
+      <c r="M30" s="50"/>
+      <c r="N30" s="50"/>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
@@ -3186,16 +3192,16 @@
     </row>
     <row r="31" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
-      <c r="B31" s="49" t="s">
+      <c r="B31" s="42" t="s">
         <v>120</v>
       </c>
-      <c r="C31" s="49" t="s">
+      <c r="C31" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="D31" s="49" t="s">
+      <c r="D31" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="E31" s="49" t="s">
+      <c r="E31" s="42" t="s">
         <v>122</v>
       </c>
       <c r="F31" s="20" t="s">
@@ -3204,25 +3210,25 @@
       <c r="G31" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="H31" s="49" t="s">
+      <c r="H31" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="I31" s="49" t="s">
+      <c r="I31" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J31" s="49" t="s">
+      <c r="J31" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="K31" s="49" t="s">
+      <c r="K31" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="L31" s="58" t="s">
+      <c r="L31" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="M31" s="49" t="s">
+      <c r="M31" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N31" s="49" t="s">
+      <c r="N31" s="42" t="s">
         <v>128</v>
       </c>
       <c r="O31" s="1"/>
@@ -3240,23 +3246,23 @@
     </row>
     <row r="32" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
-      <c r="B32" s="50"/>
-      <c r="C32" s="50"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="50"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
       <c r="F32" s="20" t="s">
         <v>129</v>
       </c>
       <c r="G32" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="H32" s="50"/>
-      <c r="I32" s="50"/>
-      <c r="J32" s="50"/>
-      <c r="K32" s="50"/>
-      <c r="L32" s="59"/>
-      <c r="M32" s="50"/>
-      <c r="N32" s="50"/>
+      <c r="H32" s="46"/>
+      <c r="I32" s="46"/>
+      <c r="J32" s="46"/>
+      <c r="K32" s="46"/>
+      <c r="L32" s="52"/>
+      <c r="M32" s="46"/>
+      <c r="N32" s="46"/>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
@@ -3272,23 +3278,23 @@
     </row>
     <row r="33" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
-      <c r="B33" s="51"/>
-      <c r="C33" s="51"/>
-      <c r="D33" s="51"/>
-      <c r="E33" s="51"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="43"/>
+      <c r="D33" s="43"/>
+      <c r="E33" s="43"/>
       <c r="F33" s="20" t="s">
         <v>131</v>
       </c>
       <c r="G33" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H33" s="51"/>
-      <c r="I33" s="51"/>
-      <c r="J33" s="51"/>
-      <c r="K33" s="51"/>
-      <c r="L33" s="60"/>
-      <c r="M33" s="51"/>
-      <c r="N33" s="51"/>
+      <c r="H33" s="43"/>
+      <c r="I33" s="43"/>
+      <c r="J33" s="43"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="53"/>
+      <c r="M33" s="43"/>
+      <c r="N33" s="43"/>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
@@ -3304,16 +3310,16 @@
     </row>
     <row r="34" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
-      <c r="B34" s="49" t="s">
+      <c r="B34" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="49" t="s">
+      <c r="C34" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="D34" s="49" t="s">
+      <c r="D34" s="42" t="s">
         <v>134</v>
       </c>
-      <c r="E34" s="49" t="s">
+      <c r="E34" s="42" t="s">
         <v>135</v>
       </c>
       <c r="F34" s="20" t="s">
@@ -3322,25 +3328,25 @@
       <c r="G34" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="H34" s="49" t="s">
+      <c r="H34" s="42" t="s">
         <v>138</v>
       </c>
-      <c r="I34" s="49" t="s">
+      <c r="I34" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="49" t="s">
+      <c r="J34" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="K34" s="49" t="s">
+      <c r="K34" s="42" t="s">
         <v>140</v>
       </c>
-      <c r="L34" s="58" t="s">
+      <c r="L34" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="M34" s="49" t="s">
+      <c r="M34" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N34" s="49" t="s">
+      <c r="N34" s="42" t="s">
         <v>141</v>
       </c>
       <c r="O34" s="1"/>
@@ -3358,23 +3364,23 @@
     </row>
     <row r="35" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
-      <c r="B35" s="50"/>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
+      <c r="B35" s="46"/>
+      <c r="C35" s="46"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="46"/>
       <c r="F35" s="20" t="s">
         <v>142</v>
       </c>
       <c r="G35" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="H35" s="50"/>
-      <c r="I35" s="50"/>
-      <c r="J35" s="50"/>
-      <c r="K35" s="50"/>
-      <c r="L35" s="59"/>
-      <c r="M35" s="50"/>
-      <c r="N35" s="50"/>
+      <c r="H35" s="46"/>
+      <c r="I35" s="46"/>
+      <c r="J35" s="46"/>
+      <c r="K35" s="46"/>
+      <c r="L35" s="52"/>
+      <c r="M35" s="46"/>
+      <c r="N35" s="46"/>
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
@@ -3390,23 +3396,23 @@
     </row>
     <row r="36" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
-      <c r="B36" s="50"/>
-      <c r="C36" s="50"/>
-      <c r="D36" s="50"/>
-      <c r="E36" s="50"/>
+      <c r="B36" s="46"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
       <c r="F36" s="20" t="s">
         <v>144</v>
       </c>
       <c r="G36" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="H36" s="50"/>
-      <c r="I36" s="50"/>
-      <c r="J36" s="50"/>
-      <c r="K36" s="50"/>
-      <c r="L36" s="59"/>
-      <c r="M36" s="50"/>
-      <c r="N36" s="50"/>
+      <c r="H36" s="46"/>
+      <c r="I36" s="46"/>
+      <c r="J36" s="46"/>
+      <c r="K36" s="46"/>
+      <c r="L36" s="52"/>
+      <c r="M36" s="46"/>
+      <c r="N36" s="46"/>
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
@@ -3422,23 +3428,23 @@
     </row>
     <row r="37" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
-      <c r="B37" s="51"/>
-      <c r="C37" s="51"/>
-      <c r="D37" s="51"/>
-      <c r="E37" s="51"/>
+      <c r="B37" s="43"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
       <c r="F37" s="20" t="s">
         <v>146</v>
       </c>
       <c r="G37" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="H37" s="51"/>
-      <c r="I37" s="51"/>
-      <c r="J37" s="51"/>
-      <c r="K37" s="51"/>
-      <c r="L37" s="60"/>
-      <c r="M37" s="51"/>
-      <c r="N37" s="51"/>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="43"/>
+      <c r="K37" s="43"/>
+      <c r="L37" s="53"/>
+      <c r="M37" s="43"/>
+      <c r="N37" s="43"/>
       <c r="O37" s="1"/>
       <c r="P37" s="1"/>
       <c r="Q37" s="1"/>
@@ -3454,16 +3460,16 @@
     </row>
     <row r="38" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
-      <c r="B38" s="49" t="s">
+      <c r="B38" s="42" t="s">
         <v>148</v>
       </c>
-      <c r="C38" s="49" t="s">
+      <c r="C38" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="D38" s="49" t="s">
+      <c r="D38" s="42" t="s">
         <v>149</v>
       </c>
-      <c r="E38" s="49" t="s">
+      <c r="E38" s="42" t="s">
         <v>150</v>
       </c>
       <c r="F38" s="20" t="s">
@@ -3472,25 +3478,25 @@
       <c r="G38" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="H38" s="49" t="s">
+      <c r="H38" s="42" t="s">
         <v>153</v>
       </c>
-      <c r="I38" s="49" t="s">
+      <c r="I38" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J38" s="49" t="s">
+      <c r="J38" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="K38" s="49" t="s">
+      <c r="K38" s="42" t="s">
         <v>154</v>
       </c>
-      <c r="L38" s="58" t="s">
+      <c r="L38" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="M38" s="49" t="s">
+      <c r="M38" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N38" s="49" t="s">
+      <c r="N38" s="42" t="s">
         <v>155</v>
       </c>
       <c r="O38" s="1"/>
@@ -3508,23 +3514,23 @@
     </row>
     <row r="39" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
-      <c r="B39" s="50"/>
-      <c r="C39" s="50"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="50"/>
+      <c r="B39" s="46"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="46"/>
+      <c r="E39" s="46"/>
       <c r="F39" s="20" t="s">
         <v>156</v>
       </c>
       <c r="G39" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="H39" s="50"/>
-      <c r="I39" s="50"/>
-      <c r="J39" s="50"/>
-      <c r="K39" s="50"/>
-      <c r="L39" s="59"/>
-      <c r="M39" s="50"/>
-      <c r="N39" s="50"/>
+      <c r="H39" s="46"/>
+      <c r="I39" s="46"/>
+      <c r="J39" s="46"/>
+      <c r="K39" s="46"/>
+      <c r="L39" s="52"/>
+      <c r="M39" s="46"/>
+      <c r="N39" s="46"/>
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
@@ -3540,23 +3546,23 @@
     </row>
     <row r="40" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
-      <c r="B40" s="51"/>
-      <c r="C40" s="51"/>
-      <c r="D40" s="51"/>
-      <c r="E40" s="51"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
       <c r="F40" s="20" t="s">
         <v>158</v>
       </c>
       <c r="G40" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="H40" s="51"/>
-      <c r="I40" s="51"/>
-      <c r="J40" s="51"/>
-      <c r="K40" s="51"/>
-      <c r="L40" s="60"/>
-      <c r="M40" s="51"/>
-      <c r="N40" s="51"/>
+      <c r="H40" s="43"/>
+      <c r="I40" s="43"/>
+      <c r="J40" s="43"/>
+      <c r="K40" s="43"/>
+      <c r="L40" s="53"/>
+      <c r="M40" s="43"/>
+      <c r="N40" s="43"/>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
@@ -3572,16 +3578,16 @@
     </row>
     <row r="41" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1"/>
-      <c r="B41" s="49" t="s">
+      <c r="B41" s="42" t="s">
         <v>160</v>
       </c>
-      <c r="C41" s="49" t="s">
+      <c r="C41" s="42" t="s">
         <v>161</v>
       </c>
-      <c r="D41" s="49" t="s">
+      <c r="D41" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="E41" s="49" t="s">
+      <c r="E41" s="42" t="s">
         <v>163</v>
       </c>
       <c r="F41" s="20" t="s">
@@ -3590,25 +3596,25 @@
       <c r="G41" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="H41" s="49" t="s">
+      <c r="H41" s="42" t="s">
         <v>166</v>
       </c>
-      <c r="I41" s="49" t="s">
+      <c r="I41" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J41" s="49" t="s">
+      <c r="J41" s="42" t="s">
         <v>167</v>
       </c>
-      <c r="K41" s="49" t="s">
+      <c r="K41" s="42" t="s">
         <v>168</v>
       </c>
-      <c r="L41" s="58" t="s">
+      <c r="L41" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="M41" s="49" t="s">
+      <c r="M41" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N41" s="49" t="s">
+      <c r="N41" s="42" t="s">
         <v>169</v>
       </c>
       <c r="O41" s="1"/>
@@ -3626,23 +3632,23 @@
     </row>
     <row r="42" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1"/>
-      <c r="B42" s="50"/>
-      <c r="C42" s="50"/>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
+      <c r="B42" s="46"/>
+      <c r="C42" s="46"/>
+      <c r="D42" s="46"/>
+      <c r="E42" s="46"/>
       <c r="F42" s="20" t="s">
         <v>170</v>
       </c>
       <c r="G42" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="H42" s="50"/>
-      <c r="I42" s="50"/>
-      <c r="J42" s="50"/>
-      <c r="K42" s="50"/>
-      <c r="L42" s="59"/>
-      <c r="M42" s="50"/>
-      <c r="N42" s="50"/>
+      <c r="H42" s="46"/>
+      <c r="I42" s="46"/>
+      <c r="J42" s="46"/>
+      <c r="K42" s="46"/>
+      <c r="L42" s="52"/>
+      <c r="M42" s="46"/>
+      <c r="N42" s="46"/>
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
@@ -3658,23 +3664,23 @@
     </row>
     <row r="43" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1"/>
-      <c r="B43" s="51"/>
-      <c r="C43" s="51"/>
-      <c r="D43" s="51"/>
-      <c r="E43" s="51"/>
+      <c r="B43" s="43"/>
+      <c r="C43" s="43"/>
+      <c r="D43" s="43"/>
+      <c r="E43" s="43"/>
       <c r="F43" s="20" t="s">
         <v>172</v>
       </c>
       <c r="G43" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="H43" s="51"/>
-      <c r="I43" s="51"/>
-      <c r="J43" s="51"/>
-      <c r="K43" s="51"/>
-      <c r="L43" s="60"/>
-      <c r="M43" s="51"/>
-      <c r="N43" s="51"/>
+      <c r="H43" s="43"/>
+      <c r="I43" s="43"/>
+      <c r="J43" s="43"/>
+      <c r="K43" s="43"/>
+      <c r="L43" s="53"/>
+      <c r="M43" s="43"/>
+      <c r="N43" s="43"/>
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
@@ -3690,16 +3696,16 @@
     </row>
     <row r="44" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1"/>
-      <c r="B44" s="49" t="s">
+      <c r="B44" s="42" t="s">
         <v>174</v>
       </c>
-      <c r="C44" s="49" t="s">
+      <c r="C44" s="42" t="s">
         <v>175</v>
       </c>
-      <c r="D44" s="49" t="s">
+      <c r="D44" s="42" t="s">
         <v>176</v>
       </c>
-      <c r="E44" s="49" t="s">
+      <c r="E44" s="42" t="s">
         <v>177</v>
       </c>
       <c r="F44" s="20" t="s">
@@ -3708,25 +3714,25 @@
       <c r="G44" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="H44" s="49" t="s">
+      <c r="H44" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="I44" s="49" t="s">
+      <c r="I44" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J44" s="49" t="s">
+      <c r="J44" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="K44" s="49" t="s">
+      <c r="K44" s="42" t="s">
         <v>182</v>
       </c>
-      <c r="L44" s="61" t="s">
+      <c r="L44" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M44" s="49" t="s">
+      <c r="M44" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N44" s="49" t="s">
+      <c r="N44" s="42" t="s">
         <v>184</v>
       </c>
       <c r="O44" s="1"/>
@@ -3744,23 +3750,23 @@
     </row>
     <row r="45" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1"/>
-      <c r="B45" s="50"/>
-      <c r="C45" s="50"/>
-      <c r="D45" s="50"/>
-      <c r="E45" s="50"/>
+      <c r="B45" s="46"/>
+      <c r="C45" s="46"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
       <c r="F45" s="20" t="s">
         <v>185</v>
       </c>
       <c r="G45" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="H45" s="50"/>
-      <c r="I45" s="50"/>
-      <c r="J45" s="50"/>
-      <c r="K45" s="50"/>
-      <c r="L45" s="62"/>
-      <c r="M45" s="50"/>
-      <c r="N45" s="50"/>
+      <c r="H45" s="46"/>
+      <c r="I45" s="46"/>
+      <c r="J45" s="46"/>
+      <c r="K45" s="46"/>
+      <c r="L45" s="47"/>
+      <c r="M45" s="46"/>
+      <c r="N45" s="46"/>
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
@@ -3776,23 +3782,23 @@
     </row>
     <row r="46" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1"/>
-      <c r="B46" s="51"/>
-      <c r="C46" s="51"/>
-      <c r="D46" s="51"/>
-      <c r="E46" s="51"/>
+      <c r="B46" s="43"/>
+      <c r="C46" s="43"/>
+      <c r="D46" s="43"/>
+      <c r="E46" s="43"/>
       <c r="F46" s="20" t="s">
         <v>187</v>
       </c>
       <c r="G46" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="H46" s="51"/>
-      <c r="I46" s="51"/>
-      <c r="J46" s="51"/>
-      <c r="K46" s="51"/>
-      <c r="L46" s="63"/>
-      <c r="M46" s="51"/>
-      <c r="N46" s="51"/>
+      <c r="H46" s="43"/>
+      <c r="I46" s="43"/>
+      <c r="J46" s="43"/>
+      <c r="K46" s="43"/>
+      <c r="L46" s="45"/>
+      <c r="M46" s="43"/>
+      <c r="N46" s="43"/>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
@@ -3808,16 +3814,16 @@
     </row>
     <row r="47" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1"/>
-      <c r="B47" s="49" t="s">
+      <c r="B47" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="C47" s="49" t="s">
+      <c r="C47" s="42" t="s">
         <v>175</v>
       </c>
-      <c r="D47" s="49" t="s">
+      <c r="D47" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="E47" s="49" t="s">
+      <c r="E47" s="42" t="s">
         <v>191</v>
       </c>
       <c r="F47" s="20" t="s">
@@ -3826,25 +3832,25 @@
       <c r="G47" s="20" t="s">
         <v>193</v>
       </c>
-      <c r="H47" s="49" t="s">
+      <c r="H47" s="42" t="s">
         <v>194</v>
       </c>
-      <c r="I47" s="49" t="s">
+      <c r="I47" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J47" s="49" t="s">
+      <c r="J47" s="42" t="s">
         <v>195</v>
       </c>
-      <c r="K47" s="49" t="s">
+      <c r="K47" s="42" t="s">
         <v>196</v>
       </c>
-      <c r="L47" s="61" t="s">
+      <c r="L47" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M47" s="49" t="s">
+      <c r="M47" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N47" s="49" t="s">
+      <c r="N47" s="42" t="s">
         <v>197</v>
       </c>
       <c r="O47" s="1"/>
@@ -3862,23 +3868,23 @@
     </row>
     <row r="48" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1"/>
-      <c r="B48" s="50"/>
-      <c r="C48" s="50"/>
-      <c r="D48" s="50"/>
-      <c r="E48" s="50"/>
+      <c r="B48" s="46"/>
+      <c r="C48" s="46"/>
+      <c r="D48" s="46"/>
+      <c r="E48" s="46"/>
       <c r="F48" s="20" t="s">
         <v>198</v>
       </c>
       <c r="G48" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="H48" s="50"/>
-      <c r="I48" s="50"/>
-      <c r="J48" s="50"/>
-      <c r="K48" s="50"/>
-      <c r="L48" s="62"/>
-      <c r="M48" s="50"/>
-      <c r="N48" s="50"/>
+      <c r="H48" s="46"/>
+      <c r="I48" s="46"/>
+      <c r="J48" s="46"/>
+      <c r="K48" s="46"/>
+      <c r="L48" s="47"/>
+      <c r="M48" s="46"/>
+      <c r="N48" s="46"/>
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
@@ -3894,23 +3900,23 @@
     </row>
     <row r="49" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1"/>
-      <c r="B49" s="51"/>
-      <c r="C49" s="51"/>
-      <c r="D49" s="51"/>
-      <c r="E49" s="51"/>
+      <c r="B49" s="43"/>
+      <c r="C49" s="43"/>
+      <c r="D49" s="43"/>
+      <c r="E49" s="43"/>
       <c r="F49" s="20" t="s">
         <v>200</v>
       </c>
       <c r="G49" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="H49" s="51"/>
-      <c r="I49" s="51"/>
-      <c r="J49" s="51"/>
-      <c r="K49" s="51"/>
-      <c r="L49" s="63"/>
-      <c r="M49" s="51"/>
-      <c r="N49" s="51"/>
+      <c r="H49" s="43"/>
+      <c r="I49" s="43"/>
+      <c r="J49" s="43"/>
+      <c r="K49" s="43"/>
+      <c r="L49" s="45"/>
+      <c r="M49" s="43"/>
+      <c r="N49" s="43"/>
       <c r="O49" s="1"/>
       <c r="P49" s="1"/>
       <c r="Q49" s="1"/>
@@ -3926,16 +3932,16 @@
     </row>
     <row r="50" spans="1:26" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1"/>
-      <c r="B50" s="49" t="s">
+      <c r="B50" s="42" t="s">
         <v>202</v>
       </c>
-      <c r="C50" s="49" t="s">
+      <c r="C50" s="42" t="s">
         <v>203</v>
       </c>
-      <c r="D50" s="49" t="s">
+      <c r="D50" s="42" t="s">
         <v>204</v>
       </c>
-      <c r="E50" s="49" t="s">
+      <c r="E50" s="42" t="s">
         <v>205</v>
       </c>
       <c r="F50" s="20" t="s">
@@ -3944,25 +3950,25 @@
       <c r="G50" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="H50" s="49" t="s">
+      <c r="H50" s="42" t="s">
         <v>208</v>
       </c>
-      <c r="I50" s="49" t="s">
+      <c r="I50" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J50" s="49" t="s">
+      <c r="J50" s="42" t="s">
         <v>209</v>
       </c>
-      <c r="K50" s="49" t="s">
+      <c r="K50" s="42" t="s">
         <v>210</v>
       </c>
-      <c r="L50" s="61" t="s">
+      <c r="L50" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M50" s="49" t="s">
+      <c r="M50" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N50" s="49" t="s">
+      <c r="N50" s="42" t="s">
         <v>211</v>
       </c>
       <c r="O50" s="1"/>
@@ -3980,23 +3986,23 @@
     </row>
     <row r="51" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1"/>
-      <c r="B51" s="51"/>
-      <c r="C51" s="51"/>
-      <c r="D51" s="51"/>
-      <c r="E51" s="51"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="43"/>
+      <c r="D51" s="43"/>
+      <c r="E51" s="43"/>
       <c r="F51" s="20" t="s">
         <v>212</v>
       </c>
       <c r="G51" s="20" t="s">
         <v>213</v>
       </c>
-      <c r="H51" s="51"/>
-      <c r="I51" s="51"/>
-      <c r="J51" s="51"/>
-      <c r="K51" s="51"/>
-      <c r="L51" s="63"/>
-      <c r="M51" s="51"/>
-      <c r="N51" s="51"/>
+      <c r="H51" s="43"/>
+      <c r="I51" s="43"/>
+      <c r="J51" s="43"/>
+      <c r="K51" s="43"/>
+      <c r="L51" s="45"/>
+      <c r="M51" s="43"/>
+      <c r="N51" s="43"/>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
@@ -4012,16 +4018,16 @@
     </row>
     <row r="52" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1"/>
-      <c r="B52" s="49" t="s">
+      <c r="B52" s="42" t="s">
         <v>214</v>
       </c>
-      <c r="C52" s="49" t="s">
+      <c r="C52" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="D52" s="49" t="s">
+      <c r="D52" s="42" t="s">
         <v>216</v>
       </c>
-      <c r="E52" s="49" t="s">
+      <c r="E52" s="42" t="s">
         <v>217</v>
       </c>
       <c r="F52" s="20" t="s">
@@ -4030,25 +4036,25 @@
       <c r="G52" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="H52" s="49" t="s">
+      <c r="H52" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="I52" s="49" t="s">
+      <c r="I52" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J52" s="49" t="s">
+      <c r="J52" s="42" t="s">
         <v>221</v>
       </c>
-      <c r="K52" s="49" t="s">
+      <c r="K52" s="42" t="s">
         <v>222</v>
       </c>
-      <c r="L52" s="61" t="s">
+      <c r="L52" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M52" s="49" t="s">
+      <c r="M52" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N52" s="49" t="s">
+      <c r="N52" s="42" t="s">
         <v>223</v>
       </c>
       <c r="O52" s="1"/>
@@ -4066,23 +4072,23 @@
     </row>
     <row r="53" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1"/>
-      <c r="B53" s="50"/>
-      <c r="C53" s="50"/>
-      <c r="D53" s="50"/>
-      <c r="E53" s="50"/>
+      <c r="B53" s="46"/>
+      <c r="C53" s="46"/>
+      <c r="D53" s="46"/>
+      <c r="E53" s="46"/>
       <c r="F53" s="20" t="s">
         <v>224</v>
       </c>
       <c r="G53" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="H53" s="50"/>
-      <c r="I53" s="50"/>
-      <c r="J53" s="50"/>
-      <c r="K53" s="50"/>
-      <c r="L53" s="62"/>
-      <c r="M53" s="50"/>
-      <c r="N53" s="50"/>
+      <c r="H53" s="46"/>
+      <c r="I53" s="46"/>
+      <c r="J53" s="46"/>
+      <c r="K53" s="46"/>
+      <c r="L53" s="47"/>
+      <c r="M53" s="46"/>
+      <c r="N53" s="46"/>
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
@@ -4098,23 +4104,23 @@
     </row>
     <row r="54" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1"/>
-      <c r="B54" s="51"/>
-      <c r="C54" s="51"/>
-      <c r="D54" s="51"/>
-      <c r="E54" s="51"/>
+      <c r="B54" s="43"/>
+      <c r="C54" s="43"/>
+      <c r="D54" s="43"/>
+      <c r="E54" s="43"/>
       <c r="F54" s="20" t="s">
         <v>226</v>
       </c>
       <c r="G54" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="H54" s="51"/>
-      <c r="I54" s="51"/>
-      <c r="J54" s="51"/>
-      <c r="K54" s="51"/>
-      <c r="L54" s="63"/>
-      <c r="M54" s="51"/>
-      <c r="N54" s="51"/>
+      <c r="H54" s="43"/>
+      <c r="I54" s="43"/>
+      <c r="J54" s="43"/>
+      <c r="K54" s="43"/>
+      <c r="L54" s="45"/>
+      <c r="M54" s="43"/>
+      <c r="N54" s="43"/>
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
@@ -4130,16 +4136,16 @@
     </row>
     <row r="55" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1"/>
-      <c r="B55" s="49" t="s">
+      <c r="B55" s="42" t="s">
         <v>228</v>
       </c>
-      <c r="C55" s="49" t="s">
+      <c r="C55" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="D55" s="49" t="s">
+      <c r="D55" s="42" t="s">
         <v>229</v>
       </c>
-      <c r="E55" s="49" t="s">
+      <c r="E55" s="42" t="s">
         <v>230</v>
       </c>
       <c r="F55" s="20" t="s">
@@ -4148,25 +4154,25 @@
       <c r="G55" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="H55" s="49" t="s">
+      <c r="H55" s="42" t="s">
         <v>233</v>
       </c>
-      <c r="I55" s="49" t="s">
+      <c r="I55" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J55" s="49" t="s">
+      <c r="J55" s="42" t="s">
         <v>234</v>
       </c>
-      <c r="K55" s="49" t="s">
+      <c r="K55" s="42" t="s">
         <v>235</v>
       </c>
-      <c r="L55" s="61" t="s">
+      <c r="L55" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M55" s="49" t="s">
+      <c r="M55" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N55" s="49" t="s">
+      <c r="N55" s="42" t="s">
         <v>236</v>
       </c>
       <c r="O55" s="1"/>
@@ -4184,23 +4190,23 @@
     </row>
     <row r="56" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1"/>
-      <c r="B56" s="51"/>
-      <c r="C56" s="51"/>
-      <c r="D56" s="51"/>
-      <c r="E56" s="51"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="43"/>
+      <c r="D56" s="43"/>
+      <c r="E56" s="43"/>
       <c r="F56" s="20" t="s">
         <v>237</v>
       </c>
       <c r="G56" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="H56" s="51"/>
-      <c r="I56" s="51"/>
-      <c r="J56" s="51"/>
-      <c r="K56" s="51"/>
-      <c r="L56" s="63"/>
-      <c r="M56" s="51"/>
-      <c r="N56" s="51"/>
+      <c r="H56" s="43"/>
+      <c r="I56" s="43"/>
+      <c r="J56" s="43"/>
+      <c r="K56" s="43"/>
+      <c r="L56" s="45"/>
+      <c r="M56" s="43"/>
+      <c r="N56" s="43"/>
       <c r="O56" s="1"/>
       <c r="P56" s="1"/>
       <c r="Q56" s="1"/>
@@ -4216,16 +4222,16 @@
     </row>
     <row r="57" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1"/>
-      <c r="B57" s="49" t="s">
+      <c r="B57" s="42" t="s">
         <v>239</v>
       </c>
-      <c r="C57" s="49" t="s">
+      <c r="C57" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="D57" s="49" t="s">
+      <c r="D57" s="42" t="s">
         <v>240</v>
       </c>
-      <c r="E57" s="49" t="s">
+      <c r="E57" s="42" t="s">
         <v>241</v>
       </c>
       <c r="F57" s="20" t="s">
@@ -4234,25 +4240,25 @@
       <c r="G57" s="20" t="s">
         <v>243</v>
       </c>
-      <c r="H57" s="49" t="s">
+      <c r="H57" s="42" t="s">
         <v>244</v>
       </c>
-      <c r="I57" s="49" t="s">
+      <c r="I57" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J57" s="49" t="s">
+      <c r="J57" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="K57" s="49" t="s">
+      <c r="K57" s="42" t="s">
         <v>245</v>
       </c>
-      <c r="L57" s="61" t="s">
+      <c r="L57" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M57" s="49" t="s">
+      <c r="M57" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N57" s="49" t="s">
+      <c r="N57" s="42" t="s">
         <v>246</v>
       </c>
       <c r="O57" s="1"/>
@@ -4270,23 +4276,23 @@
     </row>
     <row r="58" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1"/>
-      <c r="B58" s="51"/>
-      <c r="C58" s="51"/>
-      <c r="D58" s="51"/>
-      <c r="E58" s="51"/>
+      <c r="B58" s="43"/>
+      <c r="C58" s="43"/>
+      <c r="D58" s="43"/>
+      <c r="E58" s="43"/>
       <c r="F58" s="20" t="s">
         <v>247</v>
       </c>
       <c r="G58" s="20" t="s">
         <v>248</v>
       </c>
-      <c r="H58" s="51"/>
-      <c r="I58" s="51"/>
-      <c r="J58" s="51"/>
-      <c r="K58" s="51"/>
-      <c r="L58" s="63"/>
-      <c r="M58" s="51"/>
-      <c r="N58" s="51"/>
+      <c r="H58" s="43"/>
+      <c r="I58" s="43"/>
+      <c r="J58" s="43"/>
+      <c r="K58" s="43"/>
+      <c r="L58" s="45"/>
+      <c r="M58" s="43"/>
+      <c r="N58" s="43"/>
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
       <c r="Q58" s="1"/>
@@ -4302,16 +4308,16 @@
     </row>
     <row r="59" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1"/>
-      <c r="B59" s="49" t="s">
+      <c r="B59" s="42" t="s">
         <v>249</v>
       </c>
-      <c r="C59" s="49" t="s">
+      <c r="C59" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="D59" s="49" t="s">
+      <c r="D59" s="42" t="s">
         <v>250</v>
       </c>
-      <c r="E59" s="49" t="s">
+      <c r="E59" s="42" t="s">
         <v>251</v>
       </c>
       <c r="F59" s="20" t="s">
@@ -4320,25 +4326,25 @@
       <c r="G59" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="H59" s="49" t="s">
+      <c r="H59" s="42" t="s">
         <v>254</v>
       </c>
-      <c r="I59" s="49" t="s">
+      <c r="I59" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J59" s="49" t="s">
+      <c r="J59" s="42" t="s">
         <v>167</v>
       </c>
-      <c r="K59" s="49" t="s">
+      <c r="K59" s="42" t="s">
         <v>255</v>
       </c>
-      <c r="L59" s="61" t="s">
+      <c r="L59" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M59" s="49" t="s">
+      <c r="M59" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N59" s="49" t="s">
+      <c r="N59" s="42" t="s">
         <v>256</v>
       </c>
       <c r="O59" s="1"/>
@@ -4356,23 +4362,23 @@
     </row>
     <row r="60" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1"/>
-      <c r="B60" s="51"/>
-      <c r="C60" s="51"/>
-      <c r="D60" s="51"/>
-      <c r="E60" s="51"/>
+      <c r="B60" s="43"/>
+      <c r="C60" s="43"/>
+      <c r="D60" s="43"/>
+      <c r="E60" s="43"/>
       <c r="F60" s="20" t="s">
         <v>257</v>
       </c>
       <c r="G60" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="H60" s="51"/>
-      <c r="I60" s="51"/>
-      <c r="J60" s="51"/>
-      <c r="K60" s="51"/>
-      <c r="L60" s="63"/>
-      <c r="M60" s="51"/>
-      <c r="N60" s="51"/>
+      <c r="H60" s="43"/>
+      <c r="I60" s="43"/>
+      <c r="J60" s="43"/>
+      <c r="K60" s="43"/>
+      <c r="L60" s="45"/>
+      <c r="M60" s="43"/>
+      <c r="N60" s="43"/>
       <c r="O60" s="1"/>
       <c r="P60" s="1"/>
       <c r="Q60" s="1"/>
@@ -4388,16 +4394,16 @@
     </row>
     <row r="61" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1"/>
-      <c r="B61" s="49" t="s">
+      <c r="B61" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="C61" s="49" t="s">
+      <c r="C61" s="42" t="s">
         <v>260</v>
       </c>
-      <c r="D61" s="49" t="s">
+      <c r="D61" s="42" t="s">
         <v>261</v>
       </c>
-      <c r="E61" s="49" t="s">
+      <c r="E61" s="42" t="s">
         <v>262</v>
       </c>
       <c r="F61" s="20" t="s">
@@ -4406,25 +4412,25 @@
       <c r="G61" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="H61" s="49" t="s">
+      <c r="H61" s="42" t="s">
         <v>265</v>
       </c>
-      <c r="I61" s="49" t="s">
+      <c r="I61" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J61" s="49" t="s">
+      <c r="J61" s="42" t="s">
         <v>234</v>
       </c>
-      <c r="K61" s="49" t="s">
+      <c r="K61" s="42" t="s">
         <v>266</v>
       </c>
-      <c r="L61" s="61" t="s">
+      <c r="L61" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M61" s="49" t="s">
+      <c r="M61" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N61" s="49" t="s">
+      <c r="N61" s="42" t="s">
         <v>267</v>
       </c>
       <c r="O61" s="1"/>
@@ -4442,23 +4448,23 @@
     </row>
     <row r="62" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1"/>
-      <c r="B62" s="50"/>
-      <c r="C62" s="50"/>
-      <c r="D62" s="50"/>
-      <c r="E62" s="50"/>
+      <c r="B62" s="46"/>
+      <c r="C62" s="46"/>
+      <c r="D62" s="46"/>
+      <c r="E62" s="46"/>
       <c r="F62" s="20" t="s">
         <v>268</v>
       </c>
       <c r="G62" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="H62" s="50"/>
-      <c r="I62" s="50"/>
-      <c r="J62" s="50"/>
-      <c r="K62" s="50"/>
-      <c r="L62" s="62"/>
-      <c r="M62" s="50"/>
-      <c r="N62" s="50"/>
+      <c r="H62" s="46"/>
+      <c r="I62" s="46"/>
+      <c r="J62" s="46"/>
+      <c r="K62" s="46"/>
+      <c r="L62" s="47"/>
+      <c r="M62" s="46"/>
+      <c r="N62" s="46"/>
       <c r="O62" s="1"/>
       <c r="P62" s="1"/>
       <c r="Q62" s="1"/>
@@ -4474,23 +4480,23 @@
     </row>
     <row r="63" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1"/>
-      <c r="B63" s="51"/>
-      <c r="C63" s="51"/>
-      <c r="D63" s="51"/>
-      <c r="E63" s="51"/>
+      <c r="B63" s="43"/>
+      <c r="C63" s="43"/>
+      <c r="D63" s="43"/>
+      <c r="E63" s="43"/>
       <c r="F63" s="20" t="s">
         <v>270</v>
       </c>
       <c r="G63" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="H63" s="51"/>
-      <c r="I63" s="51"/>
-      <c r="J63" s="51"/>
-      <c r="K63" s="51"/>
-      <c r="L63" s="63"/>
-      <c r="M63" s="51"/>
-      <c r="N63" s="51"/>
+      <c r="H63" s="43"/>
+      <c r="I63" s="43"/>
+      <c r="J63" s="43"/>
+      <c r="K63" s="43"/>
+      <c r="L63" s="45"/>
+      <c r="M63" s="43"/>
+      <c r="N63" s="43"/>
       <c r="O63" s="1"/>
       <c r="P63" s="1"/>
       <c r="Q63" s="1"/>
@@ -4506,16 +4512,16 @@
     </row>
     <row r="64" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1"/>
-      <c r="B64" s="49" t="s">
+      <c r="B64" s="42" t="s">
         <v>272</v>
       </c>
-      <c r="C64" s="49" t="s">
+      <c r="C64" s="42" t="s">
         <v>273</v>
       </c>
-      <c r="D64" s="49" t="s">
+      <c r="D64" s="42" t="s">
         <v>274</v>
       </c>
-      <c r="E64" s="49" t="s">
+      <c r="E64" s="42" t="s">
         <v>275</v>
       </c>
       <c r="F64" s="20" t="s">
@@ -4524,25 +4530,25 @@
       <c r="G64" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="H64" s="49" t="s">
+      <c r="H64" s="42" t="s">
         <v>278</v>
       </c>
-      <c r="I64" s="49" t="s">
+      <c r="I64" s="42" t="s">
         <v>279</v>
       </c>
-      <c r="J64" s="49" t="s">
+      <c r="J64" s="42" t="s">
         <v>280</v>
       </c>
-      <c r="K64" s="49" t="s">
+      <c r="K64" s="42" t="s">
         <v>281</v>
       </c>
-      <c r="L64" s="61" t="s">
+      <c r="L64" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M64" s="49" t="s">
+      <c r="M64" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N64" s="49" t="s">
+      <c r="N64" s="42" t="s">
         <v>282</v>
       </c>
       <c r="O64" s="1"/>
@@ -4560,23 +4566,23 @@
     </row>
     <row r="65" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1"/>
-      <c r="B65" s="51"/>
-      <c r="C65" s="51"/>
-      <c r="D65" s="51"/>
-      <c r="E65" s="51"/>
+      <c r="B65" s="43"/>
+      <c r="C65" s="43"/>
+      <c r="D65" s="43"/>
+      <c r="E65" s="43"/>
       <c r="F65" s="20" t="s">
         <v>283</v>
       </c>
       <c r="G65" s="20" t="s">
         <v>284</v>
       </c>
-      <c r="H65" s="51"/>
-      <c r="I65" s="51"/>
-      <c r="J65" s="51"/>
-      <c r="K65" s="51"/>
-      <c r="L65" s="63"/>
-      <c r="M65" s="51"/>
-      <c r="N65" s="51"/>
+      <c r="H65" s="43"/>
+      <c r="I65" s="43"/>
+      <c r="J65" s="43"/>
+      <c r="K65" s="43"/>
+      <c r="L65" s="45"/>
+      <c r="M65" s="43"/>
+      <c r="N65" s="43"/>
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
       <c r="Q65" s="1"/>
@@ -4592,16 +4598,16 @@
     </row>
     <row r="66" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1"/>
-      <c r="B66" s="49" t="s">
+      <c r="B66" s="42" t="s">
         <v>285</v>
       </c>
-      <c r="C66" s="49" t="s">
+      <c r="C66" s="42" t="s">
         <v>161</v>
       </c>
-      <c r="D66" s="49" t="s">
+      <c r="D66" s="42" t="s">
         <v>286</v>
       </c>
-      <c r="E66" s="49" t="s">
+      <c r="E66" s="42" t="s">
         <v>287</v>
       </c>
       <c r="F66" s="20" t="s">
@@ -4610,25 +4616,25 @@
       <c r="G66" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="H66" s="49" t="s">
+      <c r="H66" s="42" t="s">
         <v>290</v>
       </c>
-      <c r="I66" s="49" t="s">
+      <c r="I66" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="J66" s="49" t="s">
+      <c r="J66" s="42" t="s">
         <v>291</v>
       </c>
-      <c r="K66" s="49" t="s">
+      <c r="K66" s="42" t="s">
         <v>292</v>
       </c>
-      <c r="L66" s="61" t="s">
+      <c r="L66" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="M66" s="49" t="s">
+      <c r="M66" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="N66" s="49" t="s">
+      <c r="N66" s="42" t="s">
         <v>293</v>
       </c>
       <c r="O66" s="1"/>
@@ -4646,23 +4652,23 @@
     </row>
     <row r="67" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1"/>
-      <c r="B67" s="50"/>
-      <c r="C67" s="50"/>
-      <c r="D67" s="50"/>
-      <c r="E67" s="50"/>
+      <c r="B67" s="46"/>
+      <c r="C67" s="46"/>
+      <c r="D67" s="46"/>
+      <c r="E67" s="46"/>
       <c r="F67" s="20" t="s">
         <v>294</v>
       </c>
       <c r="G67" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="H67" s="50"/>
-      <c r="I67" s="50"/>
-      <c r="J67" s="50"/>
-      <c r="K67" s="50"/>
-      <c r="L67" s="62"/>
-      <c r="M67" s="50"/>
-      <c r="N67" s="50"/>
+      <c r="H67" s="46"/>
+      <c r="I67" s="46"/>
+      <c r="J67" s="46"/>
+      <c r="K67" s="46"/>
+      <c r="L67" s="47"/>
+      <c r="M67" s="46"/>
+      <c r="N67" s="46"/>
       <c r="O67" s="1"/>
       <c r="P67" s="1"/>
       <c r="Q67" s="1"/>
@@ -4678,23 +4684,23 @@
     </row>
     <row r="68" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1"/>
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
-      <c r="D68" s="50"/>
-      <c r="E68" s="50"/>
+      <c r="B68" s="46"/>
+      <c r="C68" s="46"/>
+      <c r="D68" s="46"/>
+      <c r="E68" s="46"/>
       <c r="F68" s="20" t="s">
         <v>296</v>
       </c>
       <c r="G68" s="20" t="s">
         <v>297</v>
       </c>
-      <c r="H68" s="50"/>
-      <c r="I68" s="50"/>
-      <c r="J68" s="50"/>
-      <c r="K68" s="50"/>
-      <c r="L68" s="62"/>
-      <c r="M68" s="50"/>
-      <c r="N68" s="50"/>
+      <c r="H68" s="46"/>
+      <c r="I68" s="46"/>
+      <c r="J68" s="46"/>
+      <c r="K68" s="46"/>
+      <c r="L68" s="47"/>
+      <c r="M68" s="46"/>
+      <c r="N68" s="46"/>
       <c r="O68" s="1"/>
       <c r="P68" s="1"/>
       <c r="Q68" s="1"/>
@@ -4710,23 +4716,23 @@
     </row>
     <row r="69" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1"/>
-      <c r="B69" s="51"/>
-      <c r="C69" s="51"/>
-      <c r="D69" s="51"/>
-      <c r="E69" s="51"/>
+      <c r="B69" s="43"/>
+      <c r="C69" s="43"/>
+      <c r="D69" s="43"/>
+      <c r="E69" s="43"/>
       <c r="F69" s="20" t="s">
         <v>298</v>
       </c>
       <c r="G69" s="20" t="s">
         <v>299</v>
       </c>
-      <c r="H69" s="51"/>
-      <c r="I69" s="51"/>
-      <c r="J69" s="51"/>
-      <c r="K69" s="51"/>
-      <c r="L69" s="63"/>
-      <c r="M69" s="51"/>
-      <c r="N69" s="51"/>
+      <c r="H69" s="43"/>
+      <c r="I69" s="43"/>
+      <c r="J69" s="43"/>
+      <c r="K69" s="43"/>
+      <c r="L69" s="45"/>
+      <c r="M69" s="43"/>
+      <c r="N69" s="43"/>
       <c r="O69" s="1"/>
       <c r="P69" s="1"/>
       <c r="Q69" s="1"/>
@@ -31930,226 +31936,6 @@
     </row>
   </sheetData>
   <mergeCells count="238">
-    <mergeCell ref="K64:K65"/>
-    <mergeCell ref="L64:L65"/>
-    <mergeCell ref="M64:M65"/>
-    <mergeCell ref="N64:N65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="E64:E65"/>
-    <mergeCell ref="H64:H65"/>
-    <mergeCell ref="I64:I65"/>
-    <mergeCell ref="J64:J65"/>
-    <mergeCell ref="K61:K63"/>
-    <mergeCell ref="L61:L63"/>
-    <mergeCell ref="M61:M63"/>
-    <mergeCell ref="N61:N63"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="D61:D63"/>
-    <mergeCell ref="E61:E63"/>
-    <mergeCell ref="H61:H63"/>
-    <mergeCell ref="I61:I63"/>
-    <mergeCell ref="J61:J63"/>
-    <mergeCell ref="K59:K60"/>
-    <mergeCell ref="L59:L60"/>
-    <mergeCell ref="M59:M60"/>
-    <mergeCell ref="N59:N60"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="D59:D60"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="H59:H60"/>
-    <mergeCell ref="I59:I60"/>
-    <mergeCell ref="J59:J60"/>
-    <mergeCell ref="K57:K58"/>
-    <mergeCell ref="L57:L58"/>
-    <mergeCell ref="M57:M58"/>
-    <mergeCell ref="N57:N58"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="D57:D58"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="H57:H58"/>
-    <mergeCell ref="I57:I58"/>
-    <mergeCell ref="J57:J58"/>
-    <mergeCell ref="K55:K56"/>
-    <mergeCell ref="L55:L56"/>
-    <mergeCell ref="M55:M56"/>
-    <mergeCell ref="N55:N56"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="D55:D56"/>
-    <mergeCell ref="E55:E56"/>
-    <mergeCell ref="H55:H56"/>
-    <mergeCell ref="I55:I56"/>
-    <mergeCell ref="J55:J56"/>
-    <mergeCell ref="K52:K54"/>
-    <mergeCell ref="L52:L54"/>
-    <mergeCell ref="M52:M54"/>
-    <mergeCell ref="N52:N54"/>
-    <mergeCell ref="B52:B54"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="D52:D54"/>
-    <mergeCell ref="E52:E54"/>
-    <mergeCell ref="H52:H54"/>
-    <mergeCell ref="I52:I54"/>
-    <mergeCell ref="J52:J54"/>
-    <mergeCell ref="K50:K51"/>
-    <mergeCell ref="L50:L51"/>
-    <mergeCell ref="M50:M51"/>
-    <mergeCell ref="N50:N51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="H50:H51"/>
-    <mergeCell ref="I50:I51"/>
-    <mergeCell ref="J50:J51"/>
-    <mergeCell ref="K66:K69"/>
-    <mergeCell ref="L66:L69"/>
-    <mergeCell ref="M66:M69"/>
-    <mergeCell ref="N66:N69"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="I66:I69"/>
-    <mergeCell ref="J66:J69"/>
-    <mergeCell ref="K24:K27"/>
-    <mergeCell ref="L24:L27"/>
-    <mergeCell ref="M24:M27"/>
-    <mergeCell ref="N24:N27"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="C24:C27"/>
-    <mergeCell ref="D24:D27"/>
-    <mergeCell ref="E24:E27"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="I24:I27"/>
-    <mergeCell ref="J24:J27"/>
-    <mergeCell ref="K20:K23"/>
-    <mergeCell ref="L20:L23"/>
-    <mergeCell ref="M20:M23"/>
-    <mergeCell ref="N20:N23"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="D20:D23"/>
-    <mergeCell ref="E20:E23"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="I20:I23"/>
-    <mergeCell ref="J20:J23"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="N16:N19"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="D16:D19"/>
-    <mergeCell ref="E16:E19"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="I16:I19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="K34:K37"/>
-    <mergeCell ref="L34:L37"/>
-    <mergeCell ref="M34:M37"/>
-    <mergeCell ref="N34:N37"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="I34:I37"/>
-    <mergeCell ref="J34:J37"/>
-    <mergeCell ref="K47:K49"/>
-    <mergeCell ref="L47:L49"/>
-    <mergeCell ref="M47:M49"/>
-    <mergeCell ref="N47:N49"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="D47:D49"/>
-    <mergeCell ref="E47:E49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="I47:I49"/>
-    <mergeCell ref="J47:J49"/>
-    <mergeCell ref="K44:K46"/>
-    <mergeCell ref="L44:L46"/>
-    <mergeCell ref="M44:M46"/>
-    <mergeCell ref="N44:N46"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="D44:D46"/>
-    <mergeCell ref="E44:E46"/>
-    <mergeCell ref="H44:H46"/>
-    <mergeCell ref="I44:I46"/>
-    <mergeCell ref="J44:J46"/>
-    <mergeCell ref="K41:K43"/>
-    <mergeCell ref="L41:L43"/>
-    <mergeCell ref="M41:M43"/>
-    <mergeCell ref="N41:N43"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="D41:D43"/>
-    <mergeCell ref="E41:E43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="I41:I43"/>
-    <mergeCell ref="J41:J43"/>
-    <mergeCell ref="K38:K40"/>
-    <mergeCell ref="L38:L40"/>
-    <mergeCell ref="M38:M40"/>
-    <mergeCell ref="N38:N40"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="D38:D40"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="H38:H40"/>
-    <mergeCell ref="I38:I40"/>
-    <mergeCell ref="J38:J40"/>
-    <mergeCell ref="K31:K33"/>
-    <mergeCell ref="L31:L33"/>
-    <mergeCell ref="M31:M33"/>
-    <mergeCell ref="N31:N33"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="H31:H33"/>
-    <mergeCell ref="I31:I33"/>
-    <mergeCell ref="J31:J33"/>
-    <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="M28:M30"/>
-    <mergeCell ref="N28:N30"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="H28:H30"/>
-    <mergeCell ref="I28:I30"/>
-    <mergeCell ref="J28:J30"/>
-    <mergeCell ref="K13:K15"/>
-    <mergeCell ref="L13:L15"/>
-    <mergeCell ref="M13:M15"/>
-    <mergeCell ref="N13:N15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="H13:H15"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="J13:J15"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="B3:C3"/>
@@ -32168,6 +31954,226 @@
     <mergeCell ref="H7:H10"/>
     <mergeCell ref="I7:I10"/>
     <mergeCell ref="J7:J10"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K13:K15"/>
+    <mergeCell ref="L13:L15"/>
+    <mergeCell ref="M13:M15"/>
+    <mergeCell ref="N13:N15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="K28:K30"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="M28:M30"/>
+    <mergeCell ref="N28:N30"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="H28:H30"/>
+    <mergeCell ref="I28:I30"/>
+    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="K31:K33"/>
+    <mergeCell ref="L31:L33"/>
+    <mergeCell ref="M31:M33"/>
+    <mergeCell ref="N31:N33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="H31:H33"/>
+    <mergeCell ref="I31:I33"/>
+    <mergeCell ref="J31:J33"/>
+    <mergeCell ref="K38:K40"/>
+    <mergeCell ref="L38:L40"/>
+    <mergeCell ref="M38:M40"/>
+    <mergeCell ref="N38:N40"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="D38:D40"/>
+    <mergeCell ref="E38:E40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="I38:I40"/>
+    <mergeCell ref="J38:J40"/>
+    <mergeCell ref="K41:K43"/>
+    <mergeCell ref="L41:L43"/>
+    <mergeCell ref="M41:M43"/>
+    <mergeCell ref="N41:N43"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="D41:D43"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="I41:I43"/>
+    <mergeCell ref="J41:J43"/>
+    <mergeCell ref="K44:K46"/>
+    <mergeCell ref="L44:L46"/>
+    <mergeCell ref="M44:M46"/>
+    <mergeCell ref="N44:N46"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="D44:D46"/>
+    <mergeCell ref="E44:E46"/>
+    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="I44:I46"/>
+    <mergeCell ref="J44:J46"/>
+    <mergeCell ref="K47:K49"/>
+    <mergeCell ref="L47:L49"/>
+    <mergeCell ref="M47:M49"/>
+    <mergeCell ref="N47:N49"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="D47:D49"/>
+    <mergeCell ref="E47:E49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="I47:I49"/>
+    <mergeCell ref="J47:J49"/>
+    <mergeCell ref="K34:K37"/>
+    <mergeCell ref="L34:L37"/>
+    <mergeCell ref="M34:M37"/>
+    <mergeCell ref="N34:N37"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="I34:I37"/>
+    <mergeCell ref="J34:J37"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="N16:N19"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="D16:D19"/>
+    <mergeCell ref="E16:E19"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="I16:I19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="K20:K23"/>
+    <mergeCell ref="L20:L23"/>
+    <mergeCell ref="M20:M23"/>
+    <mergeCell ref="N20:N23"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="D20:D23"/>
+    <mergeCell ref="E20:E23"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="I20:I23"/>
+    <mergeCell ref="J20:J23"/>
+    <mergeCell ref="K24:K27"/>
+    <mergeCell ref="L24:L27"/>
+    <mergeCell ref="M24:M27"/>
+    <mergeCell ref="N24:N27"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="C24:C27"/>
+    <mergeCell ref="D24:D27"/>
+    <mergeCell ref="E24:E27"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="I24:I27"/>
+    <mergeCell ref="J24:J27"/>
+    <mergeCell ref="K66:K69"/>
+    <mergeCell ref="L66:L69"/>
+    <mergeCell ref="M66:M69"/>
+    <mergeCell ref="N66:N69"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="I66:I69"/>
+    <mergeCell ref="J66:J69"/>
+    <mergeCell ref="K50:K51"/>
+    <mergeCell ref="L50:L51"/>
+    <mergeCell ref="M50:M51"/>
+    <mergeCell ref="N50:N51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="H50:H51"/>
+    <mergeCell ref="I50:I51"/>
+    <mergeCell ref="J50:J51"/>
+    <mergeCell ref="K52:K54"/>
+    <mergeCell ref="L52:L54"/>
+    <mergeCell ref="M52:M54"/>
+    <mergeCell ref="N52:N54"/>
+    <mergeCell ref="B52:B54"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="D52:D54"/>
+    <mergeCell ref="E52:E54"/>
+    <mergeCell ref="H52:H54"/>
+    <mergeCell ref="I52:I54"/>
+    <mergeCell ref="J52:J54"/>
+    <mergeCell ref="K55:K56"/>
+    <mergeCell ref="L55:L56"/>
+    <mergeCell ref="M55:M56"/>
+    <mergeCell ref="N55:N56"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="D55:D56"/>
+    <mergeCell ref="E55:E56"/>
+    <mergeCell ref="H55:H56"/>
+    <mergeCell ref="I55:I56"/>
+    <mergeCell ref="J55:J56"/>
+    <mergeCell ref="K57:K58"/>
+    <mergeCell ref="L57:L58"/>
+    <mergeCell ref="M57:M58"/>
+    <mergeCell ref="N57:N58"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="D57:D58"/>
+    <mergeCell ref="E57:E58"/>
+    <mergeCell ref="H57:H58"/>
+    <mergeCell ref="I57:I58"/>
+    <mergeCell ref="J57:J58"/>
+    <mergeCell ref="K59:K60"/>
+    <mergeCell ref="L59:L60"/>
+    <mergeCell ref="M59:M60"/>
+    <mergeCell ref="N59:N60"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="D59:D60"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="H59:H60"/>
+    <mergeCell ref="I59:I60"/>
+    <mergeCell ref="J59:J60"/>
+    <mergeCell ref="K61:K63"/>
+    <mergeCell ref="L61:L63"/>
+    <mergeCell ref="M61:M63"/>
+    <mergeCell ref="N61:N63"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="D61:D63"/>
+    <mergeCell ref="E61:E63"/>
+    <mergeCell ref="H61:H63"/>
+    <mergeCell ref="I61:I63"/>
+    <mergeCell ref="J61:J63"/>
+    <mergeCell ref="K64:K65"/>
+    <mergeCell ref="L64:L65"/>
+    <mergeCell ref="M64:M65"/>
+    <mergeCell ref="N64:N65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="E64:E65"/>
+    <mergeCell ref="H64:H65"/>
+    <mergeCell ref="I64:I65"/>
+    <mergeCell ref="J64:J65"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:F1040 I7:N1040 G11:H1040">
     <cfRule type="expression" dxfId="24" priority="1" stopIfTrue="1">
@@ -32236,10 +32242,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I7 I11 I13 I16 I20 I24 I28 I31 I34 I38 I41 I44 I47 I50 I52 I55 I57 I59 I61 I64 I66 I70:I91" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I7 I11 I13 I16 I20 I24 I28 I31 I34 I38 I41 I44 I47 I50 I52 I55 I57 I59 I61 I64 I66 I70:I91">
       <formula1>"Alta,Medio,Bajo"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="M6:M7 M11 M13 M16 M20 M24 M28 M31 M34 M38 M41 M44 M47 M50 M52 M55 M57 M59 M61 M64 M66 M70:M119 M121:M230" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="M6:M7 M11 M13 M16 M20 M24 M28 M31 M34 M38 M41 M44 M47 M50 M52 M55 M57 M59 M61 M64 M66 M70:M119 M121:M230">
       <formula1>"Por Hacer,En Progreso,Terminado,Eliminado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -32250,7 +32256,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:J998"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -32304,11 +32310,11 @@
         <v>46125</v>
       </c>
       <c r="D3" s="31">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E3" s="32">
         <f t="shared" ref="E3:E5" si="0">IF(AND(C3&lt;&gt;"",D3&lt;&gt;""),C3+D3-1,"")</f>
-        <v>46143</v>
+        <v>46132</v>
       </c>
       <c r="F3" s="29">
         <v>18</v>
@@ -32317,7 +32323,7 @@
         <v>6</v>
       </c>
       <c r="H3" s="34">
-        <v>46145</v>
+        <v>46132</v>
       </c>
       <c r="I3" s="35" t="s">
         <v>308</v>
@@ -32329,23 +32335,23 @@
       </c>
       <c r="C4" s="36">
         <f t="shared" ref="C4:C6" si="1">IF(AND(C3&lt;&gt;"",D3&lt;&gt;"",D4&lt;&gt;""),C3+D3,"")</f>
-        <v>46144</v>
+        <v>46133</v>
       </c>
       <c r="D4" s="31">
         <v>19</v>
       </c>
       <c r="E4" s="32">
         <f t="shared" si="0"/>
-        <v>46162</v>
+        <v>46151</v>
       </c>
       <c r="F4" s="29">
         <v>29</v>
       </c>
       <c r="G4" s="33" t="s">
-        <v>305</v>
+        <v>3</v>
       </c>
       <c r="H4" s="34">
-        <v>46166</v>
+        <v>46151</v>
       </c>
       <c r="I4" s="35" t="s">
         <v>309</v>
@@ -32357,14 +32363,14 @@
       </c>
       <c r="C5" s="36">
         <f t="shared" si="1"/>
-        <v>46163</v>
+        <v>46152</v>
       </c>
       <c r="D5" s="31">
         <v>19</v>
       </c>
       <c r="E5" s="32">
         <f t="shared" si="0"/>
-        <v>46181</v>
+        <v>46170</v>
       </c>
       <c r="F5" s="29">
         <v>26</v>
@@ -32373,7 +32379,7 @@
         <v>305</v>
       </c>
       <c r="H5" s="34">
-        <v>46187</v>
+        <v>46170</v>
       </c>
       <c r="I5" s="35" t="s">
         <v>310</v>
@@ -32385,14 +32391,14 @@
       </c>
       <c r="C6" s="36">
         <f t="shared" si="1"/>
-        <v>46182</v>
+        <v>46171</v>
       </c>
       <c r="D6" s="31">
         <v>21</v>
       </c>
       <c r="E6" s="32">
         <f>IF(AND(C6&lt;&gt;"",D6&lt;&gt;""),C6+D6-1,"")</f>
-        <v>46202</v>
+        <v>46191</v>
       </c>
       <c r="F6" s="29">
         <v>61</v>
@@ -32401,7 +32407,7 @@
         <v>305</v>
       </c>
       <c r="H6" s="40">
-        <v>46208</v>
+        <v>46191</v>
       </c>
       <c r="I6" s="35" t="s">
         <v>311</v>
@@ -35622,7 +35628,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G3:G15" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G3:G15">
       <formula1>"Planeado,En Progreso,Terminado,No planeado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>